<commit_message>
feat: them ma LK-3348 (quy mo 57 model) va cap nhat ton kho chuan 100% cho toan bo danh muc
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Bang_Gia_Chuan_56_Ma" sheetId="1" r:id="rId1"/>
+    <sheet name="Bang_Gia_Chuan_57_Ma" sheetId="1" r:id="rId1"/>
     <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
     <sheet name="BienDong_Gia_NPP" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1125,25 +1125,25 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D21" t="str">
-        <v>LK-3386A</v>
+        <v>LK-3348</v>
       </c>
       <c r="E21" t="str">
-        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+        <v>Bộ nồi Táo Lock&amp;king 3 món inox cao cấp</v>
       </c>
       <c r="F21">
-        <v>550000</v>
+        <v>580000</v>
       </c>
       <c r="G21">
-        <v>990000</v>
+        <v>1044000</v>
       </c>
       <c r="H21">
-        <v>1040000</v>
+        <v>1097000</v>
       </c>
       <c r="I21">
-        <v>1248000</v>
+        <v>1317000</v>
       </c>
       <c r="J21">
-        <v>440000</v>
+        <v>464000</v>
       </c>
       <c r="K21" t="str">
         <v>44.4%</v>
@@ -1160,28 +1160,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D22" t="str">
-        <v>LK-3568A</v>
+        <v>LK-3386A</v>
       </c>
       <c r="E22" t="str">
-        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
       </c>
       <c r="F22">
-        <v>960000</v>
+        <v>550000</v>
       </c>
       <c r="G22">
-        <v>1690000</v>
+        <v>990000</v>
       </c>
       <c r="H22">
-        <v>1775000</v>
+        <v>1040000</v>
       </c>
       <c r="I22">
-        <v>2130000</v>
+        <v>1248000</v>
       </c>
       <c r="J22">
-        <v>730000</v>
+        <v>440000</v>
       </c>
       <c r="K22" t="str">
-        <v>43.2%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="23">
@@ -1192,31 +1192,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C23" t="str">
-        <v>NỒI TĂNG ÁP</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D23" t="str">
-        <v>LK-3122</v>
+        <v>LK-3568A</v>
       </c>
       <c r="E23" t="str">
-        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
       </c>
       <c r="F23">
-        <v>470000</v>
+        <v>960000</v>
       </c>
       <c r="G23">
-        <v>820000</v>
+        <v>1690000</v>
       </c>
       <c r="H23">
-        <v>886000</v>
+        <v>1775000</v>
       </c>
       <c r="I23">
-        <v>1064000</v>
+        <v>2130000</v>
       </c>
       <c r="J23">
-        <v>350000</v>
+        <v>730000</v>
       </c>
       <c r="K23" t="str">
-        <v>42.7%</v>
+        <v>43.2%</v>
       </c>
     </row>
     <row r="24">
@@ -1230,28 +1230,28 @@
         <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D24" t="str">
-        <v>LK-3126</v>
+        <v>LK-3122</v>
       </c>
       <c r="E24" t="str">
-        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
       </c>
       <c r="F24">
-        <v>535000</v>
+        <v>470000</v>
       </c>
       <c r="G24">
-        <v>990000</v>
+        <v>820000</v>
       </c>
       <c r="H24">
-        <v>1070000</v>
+        <v>886000</v>
       </c>
       <c r="I24">
-        <v>1284000</v>
+        <v>1064000</v>
       </c>
       <c r="J24">
-        <v>455000</v>
+        <v>350000</v>
       </c>
       <c r="K24" t="str">
-        <v>46.0%</v>
+        <v>42.7%</v>
       </c>
     </row>
     <row r="25">
@@ -1262,31 +1262,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C25" t="str">
-        <v>ẤM &amp; BÌNH</v>
+        <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D25" t="str">
-        <v>LK-1038</v>
+        <v>LK-3126</v>
       </c>
       <c r="E25" t="str">
-        <v>Ấm đun nước LK-1038</v>
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
       </c>
       <c r="F25">
-        <v>300000</v>
+        <v>535000</v>
       </c>
       <c r="G25">
-        <v>525000</v>
+        <v>990000</v>
       </c>
       <c r="H25">
-        <v>552000</v>
+        <v>1070000</v>
       </c>
       <c r="I25">
-        <v>663000</v>
+        <v>1284000</v>
       </c>
       <c r="J25">
-        <v>225000</v>
+        <v>455000</v>
       </c>
       <c r="K25" t="str">
-        <v>42.9%</v>
+        <v>46.0%</v>
       </c>
     </row>
     <row r="26">
@@ -1297,31 +1297,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C26" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>ẤM &amp; BÌNH</v>
       </c>
       <c r="D26" t="str">
-        <v>LK-92</v>
+        <v>LK-1038</v>
       </c>
       <c r="E26" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Ấm đun nước LK-1038</v>
       </c>
       <c r="F26">
-        <v>835000</v>
+        <v>300000</v>
       </c>
       <c r="G26">
-        <v>1590000</v>
+        <v>525000</v>
       </c>
       <c r="H26">
-        <v>1670000</v>
+        <v>552000</v>
       </c>
       <c r="I26">
-        <v>2004000</v>
+        <v>663000</v>
       </c>
       <c r="J26">
-        <v>755000</v>
+        <v>225000</v>
       </c>
       <c r="K26" t="str">
-        <v>47.5%</v>
+        <v>42.9%</v>
       </c>
     </row>
     <row r="27">
@@ -1335,28 +1335,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D27" t="str">
-        <v>LK-586</v>
+        <v>LK-92</v>
       </c>
       <c r="E27" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F27">
-        <v>430000</v>
+        <v>835000</v>
       </c>
       <c r="G27">
-        <v>745000</v>
+        <v>1590000</v>
       </c>
       <c r="H27">
-        <v>783000</v>
+        <v>1670000</v>
       </c>
       <c r="I27">
-        <v>940000</v>
+        <v>2004000</v>
       </c>
       <c r="J27">
-        <v>315000</v>
+        <v>755000</v>
       </c>
       <c r="K27" t="str">
-        <v>42.3%</v>
+        <v>47.5%</v>
       </c>
     </row>
     <row r="28">
@@ -1370,28 +1370,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D28" t="str">
-        <v>LK-588</v>
+        <v>LK-586</v>
       </c>
       <c r="E28" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F28">
-        <v>585000</v>
+        <v>430000</v>
       </c>
       <c r="G28">
-        <v>1050000</v>
+        <v>745000</v>
       </c>
       <c r="H28">
-        <v>1103000</v>
+        <v>783000</v>
       </c>
       <c r="I28">
-        <v>1324000</v>
+        <v>940000</v>
       </c>
       <c r="J28">
-        <v>465000</v>
+        <v>315000</v>
       </c>
       <c r="K28" t="str">
-        <v>44.3%</v>
+        <v>42.3%</v>
       </c>
     </row>
     <row r="29">
@@ -1405,28 +1405,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D29" t="str">
-        <v>LK-668</v>
+        <v>LK-588</v>
       </c>
       <c r="E29" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F29">
-        <v>460000</v>
+        <v>585000</v>
       </c>
       <c r="G29">
-        <v>920000</v>
+        <v>1050000</v>
       </c>
       <c r="H29">
-        <v>966000</v>
+        <v>1103000</v>
       </c>
       <c r="I29">
-        <v>1160000</v>
+        <v>1324000</v>
       </c>
       <c r="J29">
-        <v>460000</v>
+        <v>465000</v>
       </c>
       <c r="K29" t="str">
-        <v>50.0%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="30">
@@ -1440,28 +1440,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D30" t="str">
-        <v>LK-688</v>
+        <v>LK-668</v>
       </c>
       <c r="E30" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
       </c>
       <c r="F30">
-        <v>850000</v>
+        <v>460000</v>
       </c>
       <c r="G30">
-        <v>1690000</v>
+        <v>920000</v>
       </c>
       <c r="H30">
-        <v>1775000</v>
+        <v>966000</v>
       </c>
       <c r="I30">
-        <v>2130000</v>
+        <v>1160000</v>
       </c>
       <c r="J30">
-        <v>840000</v>
+        <v>460000</v>
       </c>
       <c r="K30" t="str">
-        <v>49.7%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="31">
@@ -1475,28 +1475,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D31" t="str">
-        <v>LK-1003</v>
+        <v>LK-688</v>
       </c>
       <c r="E31" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
       </c>
       <c r="F31">
-        <v>197000</v>
+        <v>850000</v>
       </c>
       <c r="G31">
-        <v>354000</v>
+        <v>1690000</v>
       </c>
       <c r="H31">
-        <v>372000</v>
+        <v>1775000</v>
       </c>
       <c r="I31">
-        <v>447000</v>
+        <v>2130000</v>
       </c>
       <c r="J31">
-        <v>157000</v>
+        <v>840000</v>
       </c>
       <c r="K31" t="str">
-        <v>44.4%</v>
+        <v>49.7%</v>
       </c>
     </row>
     <row r="32">
@@ -1510,28 +1510,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E32" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F32">
-        <v>1020000</v>
+        <v>197000</v>
       </c>
       <c r="G32">
-        <v>1890000</v>
+        <v>354000</v>
       </c>
       <c r="H32">
-        <v>1985000</v>
+        <v>372000</v>
       </c>
       <c r="I32">
-        <v>2382000</v>
+        <v>447000</v>
       </c>
       <c r="J32">
-        <v>870000</v>
+        <v>157000</v>
       </c>
       <c r="K32" t="str">
-        <v>46.0%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="33">
@@ -1545,28 +1545,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E33" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F33">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="G33">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="H33">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
       <c r="I33">
-        <v>845000</v>
+        <v>2382000</v>
       </c>
       <c r="J33">
-        <v>298000</v>
+        <v>870000</v>
       </c>
       <c r="K33" t="str">
-        <v>44.5%</v>
+        <v>46.0%</v>
       </c>
     </row>
     <row r="34">
@@ -1580,28 +1580,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E34" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F34">
-        <v>780000</v>
+        <v>372000</v>
       </c>
       <c r="G34">
-        <v>1495000</v>
+        <v>670000</v>
       </c>
       <c r="H34">
-        <v>1570000</v>
+        <v>704000</v>
       </c>
       <c r="I34">
-        <v>1884000</v>
+        <v>845000</v>
       </c>
       <c r="J34">
-        <v>715000</v>
+        <v>298000</v>
       </c>
       <c r="K34" t="str">
-        <v>47.8%</v>
+        <v>44.5%</v>
       </c>
     </row>
     <row r="35">
@@ -1615,28 +1615,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E35" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F35">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="G35">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="H35">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
       <c r="I35">
-        <v>755000</v>
+        <v>1884000</v>
       </c>
       <c r="J35">
-        <v>289000</v>
+        <v>715000</v>
       </c>
       <c r="K35" t="str">
-        <v>48.2%</v>
+        <v>47.8%</v>
       </c>
     </row>
     <row r="36">
@@ -1650,28 +1650,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E36" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F36">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="G36">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="H36">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
       <c r="I36">
-        <v>2369000</v>
+        <v>755000</v>
       </c>
       <c r="J36">
-        <v>880000</v>
+        <v>289000</v>
       </c>
       <c r="K36" t="str">
-        <v>46.8%</v>
+        <v>48.2%</v>
       </c>
     </row>
     <row r="37">
@@ -1685,28 +1685,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F37">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="G37">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="H37">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
       <c r="I37">
-        <v>1878000</v>
+        <v>2369000</v>
       </c>
       <c r="J37">
-        <v>690000</v>
+        <v>880000</v>
       </c>
       <c r="K37" t="str">
-        <v>46.3%</v>
+        <v>46.8%</v>
       </c>
     </row>
     <row r="38">
@@ -1720,25 +1720,25 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F38">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="G38">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="H38">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
       <c r="I38">
-        <v>1198000</v>
+        <v>1878000</v>
       </c>
       <c r="J38">
-        <v>440000</v>
+        <v>690000</v>
       </c>
       <c r="K38" t="str">
         <v>46.3%</v>
@@ -1755,10 +1755,10 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F39">
         <v>510000</v>
@@ -1790,28 +1790,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E40" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F40">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="G40">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="H40">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
       <c r="I40">
-        <v>1500000</v>
+        <v>1198000</v>
       </c>
       <c r="J40">
-        <v>590000</v>
+        <v>440000</v>
       </c>
       <c r="K40" t="str">
-        <v>49.6%</v>
+        <v>46.3%</v>
       </c>
     </row>
     <row r="41">
@@ -1825,28 +1825,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E41" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F41">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="G41">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="H41">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
       <c r="I41">
-        <v>618000</v>
+        <v>1500000</v>
       </c>
       <c r="J41">
-        <v>230000</v>
+        <v>590000</v>
       </c>
       <c r="K41" t="str">
-        <v>46.9%</v>
+        <v>49.6%</v>
       </c>
     </row>
     <row r="42">
@@ -1860,25 +1860,25 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F42">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="G42">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="H42">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
       <c r="I42">
-        <v>1626000</v>
+        <v>618000</v>
       </c>
       <c r="J42">
-        <v>605000</v>
+        <v>230000</v>
       </c>
       <c r="K42" t="str">
         <v>46.9%</v>
@@ -1895,28 +1895,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E43" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F43">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="G43">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="H43">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
       <c r="I43">
-        <v>1500000</v>
+        <v>1626000</v>
       </c>
       <c r="J43">
-        <v>530000</v>
+        <v>605000</v>
       </c>
       <c r="K43" t="str">
-        <v>44.5%</v>
+        <v>46.9%</v>
       </c>
     </row>
     <row r="44">
@@ -1930,28 +1930,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E44" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F44">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="G44">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="H44">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
       <c r="I44">
-        <v>2760000</v>
+        <v>1500000</v>
       </c>
       <c r="J44">
-        <v>1060000</v>
+        <v>530000</v>
       </c>
       <c r="K44" t="str">
-        <v>48.4%</v>
+        <v>44.5%</v>
       </c>
     </row>
     <row r="45">
@@ -1959,34 +1959,34 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C45" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E45" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F45">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="G45">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="H45">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
       <c r="I45">
-        <v>590000</v>
+        <v>2760000</v>
       </c>
       <c r="J45">
-        <v>202000</v>
+        <v>1060000</v>
       </c>
       <c r="K45" t="str">
-        <v>43.3%</v>
+        <v>48.4%</v>
       </c>
     </row>
     <row r="46">
@@ -2000,28 +2000,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2662</v>
+        <v>TK-2201</v>
       </c>
       <c r="E46" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F46">
-        <v>320000</v>
+        <v>265000</v>
       </c>
       <c r="G46">
+        <v>467000</v>
+      </c>
+      <c r="H46">
+        <v>491000</v>
+      </c>
+      <c r="I46">
         <v>590000</v>
       </c>
-      <c r="H46">
-        <v>620000</v>
-      </c>
-      <c r="I46">
-        <v>744000</v>
-      </c>
       <c r="J46">
-        <v>270000</v>
+        <v>202000</v>
       </c>
       <c r="K46" t="str">
-        <v>45.8%</v>
+        <v>43.3%</v>
       </c>
     </row>
     <row r="47">
@@ -2035,28 +2035,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2882C</v>
+        <v>TK-2662</v>
       </c>
       <c r="E47" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F47">
-        <v>351000</v>
+        <v>320000</v>
       </c>
       <c r="G47">
-        <v>630000</v>
+        <v>590000</v>
       </c>
       <c r="H47">
-        <v>662000</v>
+        <v>620000</v>
       </c>
       <c r="I47">
-        <v>795000</v>
+        <v>744000</v>
       </c>
       <c r="J47">
-        <v>279000</v>
+        <v>270000</v>
       </c>
       <c r="K47" t="str">
-        <v>44.3%</v>
+        <v>45.8%</v>
       </c>
     </row>
     <row r="48">
@@ -2070,28 +2070,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-3030C</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F48">
-        <v>375000</v>
+        <v>351000</v>
       </c>
       <c r="G48">
-        <v>750000</v>
+        <v>630000</v>
       </c>
       <c r="H48">
-        <v>788000</v>
+        <v>662000</v>
       </c>
       <c r="I48">
-        <v>946000</v>
+        <v>795000</v>
       </c>
       <c r="J48">
-        <v>375000</v>
+        <v>279000</v>
       </c>
       <c r="K48" t="str">
-        <v>50.0%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="49">
@@ -2102,31 +2102,31 @@
         <v>Takin</v>
       </c>
       <c r="C49" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-036A</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E49" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F49">
-        <v>515000</v>
+        <v>375000</v>
       </c>
       <c r="G49">
-        <v>891000</v>
+        <v>750000</v>
       </c>
       <c r="H49">
-        <v>936000</v>
+        <v>788000</v>
       </c>
       <c r="I49">
-        <v>1124000</v>
+        <v>946000</v>
       </c>
       <c r="J49">
-        <v>376000</v>
+        <v>375000</v>
       </c>
       <c r="K49" t="str">
-        <v>42.2%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="50">
@@ -2140,28 +2140,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-0324</v>
+        <v>TK-036A</v>
       </c>
       <c r="E50" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F50">
-        <v>245000</v>
+        <v>515000</v>
       </c>
       <c r="G50">
-        <v>441000</v>
+        <v>891000</v>
       </c>
       <c r="H50">
-        <v>464000</v>
+        <v>936000</v>
       </c>
       <c r="I50">
-        <v>557000</v>
+        <v>1124000</v>
       </c>
       <c r="J50">
-        <v>196000</v>
+        <v>376000</v>
       </c>
       <c r="K50" t="str">
-        <v>44.4%</v>
+        <v>42.2%</v>
       </c>
     </row>
     <row r="51">
@@ -2175,25 +2175,25 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0348A</v>
+        <v>TK-0324</v>
       </c>
       <c r="E51" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F51">
-        <v>580000</v>
+        <v>245000</v>
       </c>
       <c r="G51">
-        <v>1044000</v>
+        <v>441000</v>
       </c>
       <c r="H51">
-        <v>1097000</v>
+        <v>464000</v>
       </c>
       <c r="I51">
-        <v>1317000</v>
+        <v>557000</v>
       </c>
       <c r="J51">
-        <v>464000</v>
+        <v>196000</v>
       </c>
       <c r="K51" t="str">
         <v>44.4%</v>
@@ -2210,28 +2210,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0369</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F52">
-        <v>535000</v>
+        <v>580000</v>
       </c>
       <c r="G52">
-        <v>969000</v>
+        <v>1044000</v>
       </c>
       <c r="H52">
-        <v>1018000</v>
+        <v>1097000</v>
       </c>
       <c r="I52">
-        <v>1222000</v>
+        <v>1317000</v>
       </c>
       <c r="J52">
-        <v>434000</v>
+        <v>464000</v>
       </c>
       <c r="K52" t="str">
-        <v>44.8%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="53">
@@ -2245,28 +2245,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0488</v>
+        <v>TK-0369</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F53">
-        <v>810000</v>
+        <v>535000</v>
       </c>
       <c r="G53">
-        <v>1469000</v>
+        <v>969000</v>
       </c>
       <c r="H53">
-        <v>1543000</v>
+        <v>1018000</v>
       </c>
       <c r="I53">
-        <v>1852000</v>
+        <v>1222000</v>
       </c>
       <c r="J53">
-        <v>659000</v>
+        <v>434000</v>
       </c>
       <c r="K53" t="str">
-        <v>44.9%</v>
+        <v>44.8%</v>
       </c>
     </row>
     <row r="54">
@@ -2277,31 +2277,31 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-468</v>
+        <v>TK-0488</v>
       </c>
       <c r="E54" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F54">
-        <v>452000</v>
+        <v>810000</v>
       </c>
       <c r="G54">
-        <v>900000</v>
+        <v>1469000</v>
       </c>
       <c r="H54">
-        <v>945000</v>
+        <v>1543000</v>
       </c>
       <c r="I54">
-        <v>1134000</v>
+        <v>1852000</v>
       </c>
       <c r="J54">
-        <v>448000</v>
+        <v>659000</v>
       </c>
       <c r="K54" t="str">
-        <v>49.8%</v>
+        <v>44.9%</v>
       </c>
     </row>
     <row r="55">
@@ -2315,28 +2315,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-469</v>
+        <v>TK-468</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F55">
-        <v>615000</v>
+        <v>452000</v>
       </c>
       <c r="G55">
-        <v>1050000</v>
+        <v>900000</v>
       </c>
       <c r="H55">
-        <v>1103000</v>
+        <v>945000</v>
       </c>
       <c r="I55">
-        <v>1324000</v>
+        <v>1134000</v>
       </c>
       <c r="J55">
-        <v>435000</v>
+        <v>448000</v>
       </c>
       <c r="K55" t="str">
-        <v>41.4%</v>
+        <v>49.8%</v>
       </c>
     </row>
     <row r="56">
@@ -2350,28 +2350,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-1002</v>
+        <v>TK-469</v>
       </c>
       <c r="E56" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F56">
-        <v>158000</v>
+        <v>615000</v>
       </c>
       <c r="G56">
-        <v>270000</v>
+        <v>1050000</v>
       </c>
       <c r="H56">
-        <v>284000</v>
+        <v>1103000</v>
       </c>
       <c r="I56">
-        <v>341000</v>
+        <v>1324000</v>
       </c>
       <c r="J56">
-        <v>112000</v>
+        <v>435000</v>
       </c>
       <c r="K56" t="str">
-        <v>41.5%</v>
+        <v>41.4%</v>
       </c>
     </row>
     <row r="57">
@@ -2385,40 +2385,75 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D57" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F57">
+        <v>158000</v>
+      </c>
+      <c r="G57">
+        <v>270000</v>
+      </c>
+      <c r="H57">
+        <v>284000</v>
+      </c>
+      <c r="I57">
+        <v>341000</v>
+      </c>
+      <c r="J57">
+        <v>112000</v>
+      </c>
+      <c r="K57" t="str">
+        <v>41.5%</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C58" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D58" t="str">
         <v>TK-1003</v>
       </c>
-      <c r="E57" t="str">
+      <c r="E58" t="str">
         <v>Bộ đèn sưởi 3 bóng Takin</v>
       </c>
-      <c r="F57">
+      <c r="F58">
         <v>194000</v>
       </c>
-      <c r="G57">
+      <c r="G58">
         <v>330000</v>
       </c>
-      <c r="H57">
+      <c r="H58">
         <v>347000</v>
       </c>
-      <c r="I57">
+      <c r="I58">
         <v>417000</v>
       </c>
-      <c r="J57">
+      <c r="J58">
         <v>136000</v>
       </c>
-      <c r="K57" t="str">
+      <c r="K58" t="str">
         <v>41.2%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K58"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N58"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -3329,37 +3364,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D21" t="str">
-        <v>LK-3386A</v>
+        <v>LK-3348</v>
       </c>
       <c r="E21" t="str">
-        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+        <v>Bộ nồi Táo Lock&amp;king 3 món inox cao cấp</v>
       </c>
       <c r="F21">
-        <v>453015</v>
+        <v>474876</v>
       </c>
       <c r="G21">
-        <v>550000</v>
+        <v>580000</v>
       </c>
       <c r="H21">
-        <v>990000</v>
+        <v>1044000</v>
       </c>
       <c r="I21">
-        <v>440000</v>
+        <v>464000</v>
       </c>
       <c r="J21" t="str">
         <v>44.4%</v>
       </c>
       <c r="K21">
-        <v>1040000</v>
+        <v>1097000</v>
       </c>
       <c r="L21">
-        <v>50000</v>
+        <v>53000</v>
       </c>
       <c r="M21" t="str">
         <v>5.1%</v>
       </c>
       <c r="N21">
-        <v>1248000</v>
+        <v>1317000</v>
       </c>
     </row>
     <row r="22">
@@ -3373,37 +3408,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D22" t="str">
-        <v>LK-3568A</v>
+        <v>LK-3386A</v>
       </c>
       <c r="E22" t="str">
-        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
       </c>
       <c r="F22">
-        <v>815667</v>
+        <v>453015</v>
       </c>
       <c r="G22">
-        <v>960000</v>
+        <v>550000</v>
       </c>
       <c r="H22">
-        <v>1690000</v>
+        <v>990000</v>
       </c>
       <c r="I22">
-        <v>730000</v>
+        <v>440000</v>
       </c>
       <c r="J22" t="str">
-        <v>43.2%</v>
+        <v>44.4%</v>
       </c>
       <c r="K22">
-        <v>1775000</v>
+        <v>1040000</v>
       </c>
       <c r="L22">
-        <v>85000</v>
+        <v>50000</v>
       </c>
       <c r="M22" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N22">
-        <v>2130000</v>
+        <v>1248000</v>
       </c>
     </row>
     <row r="23">
@@ -3414,40 +3449,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C23" t="str">
-        <v>NỒI TĂNG ÁP</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D23" t="str">
-        <v>LK-3122</v>
+        <v>LK-3568A</v>
       </c>
       <c r="E23" t="str">
-        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
       </c>
       <c r="F23">
-        <v>357441</v>
+        <v>815667</v>
       </c>
       <c r="G23">
-        <v>470000</v>
+        <v>960000</v>
       </c>
       <c r="H23">
-        <v>820000</v>
+        <v>1690000</v>
       </c>
       <c r="I23">
-        <v>350000</v>
+        <v>730000</v>
       </c>
       <c r="J23" t="str">
-        <v>42.7%</v>
+        <v>43.2%</v>
       </c>
       <c r="K23">
-        <v>886000</v>
+        <v>1775000</v>
       </c>
       <c r="L23">
-        <v>66000</v>
+        <v>85000</v>
       </c>
       <c r="M23" t="str">
-        <v>8.0%</v>
+        <v>5.0%</v>
       </c>
       <c r="N23">
-        <v>1064000</v>
+        <v>2130000</v>
       </c>
     </row>
     <row r="24">
@@ -3461,37 +3496,37 @@
         <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D24" t="str">
-        <v>LK-3126</v>
+        <v>LK-3122</v>
       </c>
       <c r="E24" t="str">
-        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
       </c>
       <c r="F24">
-        <v>387848</v>
+        <v>357441</v>
       </c>
       <c r="G24">
-        <v>535000</v>
+        <v>470000</v>
       </c>
       <c r="H24">
-        <v>990000</v>
+        <v>820000</v>
       </c>
       <c r="I24">
-        <v>455000</v>
+        <v>350000</v>
       </c>
       <c r="J24" t="str">
-        <v>46.0%</v>
+        <v>42.7%</v>
       </c>
       <c r="K24">
-        <v>1070000</v>
+        <v>886000</v>
       </c>
       <c r="L24">
-        <v>80000</v>
+        <v>66000</v>
       </c>
       <c r="M24" t="str">
-        <v>8.1%</v>
+        <v>8.0%</v>
       </c>
       <c r="N24">
-        <v>1284000</v>
+        <v>1064000</v>
       </c>
     </row>
     <row r="25">
@@ -3502,40 +3537,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C25" t="str">
-        <v>ẤM &amp; BÌNH</v>
+        <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D25" t="str">
-        <v>LK-1038</v>
+        <v>LK-3126</v>
       </c>
       <c r="E25" t="str">
-        <v>Ấm đun nước LK-1038</v>
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
       </c>
       <c r="F25">
-        <v>235094</v>
+        <v>387848</v>
       </c>
       <c r="G25">
-        <v>300000</v>
+        <v>535000</v>
       </c>
       <c r="H25">
-        <v>525000</v>
+        <v>990000</v>
       </c>
       <c r="I25">
-        <v>225000</v>
+        <v>455000</v>
       </c>
       <c r="J25" t="str">
-        <v>42.9%</v>
+        <v>46.0%</v>
       </c>
       <c r="K25">
-        <v>552000</v>
+        <v>1070000</v>
       </c>
       <c r="L25">
-        <v>27000</v>
+        <v>80000</v>
       </c>
       <c r="M25" t="str">
-        <v>5.1%</v>
+        <v>8.1%</v>
       </c>
       <c r="N25">
-        <v>663000</v>
+        <v>1284000</v>
       </c>
     </row>
     <row r="26">
@@ -3546,40 +3581,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C26" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>ẤM &amp; BÌNH</v>
       </c>
       <c r="D26" t="str">
-        <v>LK-92</v>
+        <v>LK-1038</v>
       </c>
       <c r="E26" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Ấm đun nước LK-1038</v>
       </c>
       <c r="F26">
-        <v>727600</v>
+        <v>235094</v>
       </c>
       <c r="G26">
-        <v>835000</v>
+        <v>300000</v>
       </c>
       <c r="H26">
-        <v>1590000</v>
+        <v>525000</v>
       </c>
       <c r="I26">
-        <v>755000</v>
+        <v>225000</v>
       </c>
       <c r="J26" t="str">
-        <v>47.5%</v>
+        <v>42.9%</v>
       </c>
       <c r="K26">
-        <v>1670000</v>
+        <v>552000</v>
       </c>
       <c r="L26">
-        <v>80000</v>
+        <v>27000</v>
       </c>
       <c r="M26" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N26">
-        <v>2004000</v>
+        <v>663000</v>
       </c>
     </row>
     <row r="27">
@@ -3593,37 +3628,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D27" t="str">
-        <v>LK-586</v>
+        <v>LK-92</v>
       </c>
       <c r="E27" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F27">
-        <v>366857</v>
+        <v>727600</v>
       </c>
       <c r="G27">
-        <v>430000</v>
+        <v>835000</v>
       </c>
       <c r="H27">
-        <v>745000</v>
+        <v>1590000</v>
       </c>
       <c r="I27">
-        <v>315000</v>
+        <v>755000</v>
       </c>
       <c r="J27" t="str">
-        <v>42.3%</v>
+        <v>47.5%</v>
       </c>
       <c r="K27">
-        <v>783000</v>
+        <v>1670000</v>
       </c>
       <c r="L27">
-        <v>38000</v>
+        <v>80000</v>
       </c>
       <c r="M27" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N27">
-        <v>940000</v>
+        <v>2004000</v>
       </c>
     </row>
     <row r="28">
@@ -3637,37 +3672,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D28" t="str">
-        <v>LK-588</v>
+        <v>LK-586</v>
       </c>
       <c r="E28" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F28">
-        <v>468762</v>
+        <v>366857</v>
       </c>
       <c r="G28">
-        <v>585000</v>
+        <v>430000</v>
       </c>
       <c r="H28">
-        <v>1050000</v>
+        <v>745000</v>
       </c>
       <c r="I28">
-        <v>465000</v>
+        <v>315000</v>
       </c>
       <c r="J28" t="str">
-        <v>44.3%</v>
+        <v>42.3%</v>
       </c>
       <c r="K28">
-        <v>1103000</v>
+        <v>783000</v>
       </c>
       <c r="L28">
-        <v>53000</v>
+        <v>38000</v>
       </c>
       <c r="M28" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N28">
-        <v>1324000</v>
+        <v>940000</v>
       </c>
     </row>
     <row r="29">
@@ -3681,37 +3716,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D29" t="str">
-        <v>LK-668</v>
+        <v>LK-588</v>
       </c>
       <c r="E29" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F29">
-        <v>395900</v>
+        <v>468762</v>
       </c>
       <c r="G29">
-        <v>460000</v>
+        <v>585000</v>
       </c>
       <c r="H29">
-        <v>920000</v>
+        <v>1050000</v>
       </c>
       <c r="I29">
-        <v>460000</v>
+        <v>465000</v>
       </c>
       <c r="J29" t="str">
-        <v>50.0%</v>
+        <v>44.3%</v>
       </c>
       <c r="K29">
-        <v>966000</v>
+        <v>1103000</v>
       </c>
       <c r="L29">
-        <v>46000</v>
+        <v>53000</v>
       </c>
       <c r="M29" t="str">
         <v>5.0%</v>
       </c>
       <c r="N29">
-        <v>1160000</v>
+        <v>1324000</v>
       </c>
     </row>
     <row r="30">
@@ -3725,37 +3760,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D30" t="str">
-        <v>LK-688</v>
+        <v>LK-668</v>
       </c>
       <c r="E30" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
       </c>
       <c r="F30">
-        <v>727600</v>
+        <v>395900</v>
       </c>
       <c r="G30">
-        <v>850000</v>
+        <v>460000</v>
       </c>
       <c r="H30">
-        <v>1690000</v>
+        <v>920000</v>
       </c>
       <c r="I30">
-        <v>840000</v>
+        <v>460000</v>
       </c>
       <c r="J30" t="str">
-        <v>49.7%</v>
+        <v>50.0%</v>
       </c>
       <c r="K30">
-        <v>1775000</v>
+        <v>966000</v>
       </c>
       <c r="L30">
-        <v>85000</v>
+        <v>46000</v>
       </c>
       <c r="M30" t="str">
         <v>5.0%</v>
       </c>
       <c r="N30">
-        <v>2130000</v>
+        <v>1160000</v>
       </c>
     </row>
     <row r="31">
@@ -3769,37 +3804,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D31" t="str">
-        <v>LK-1003</v>
+        <v>LK-688</v>
       </c>
       <c r="E31" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
       </c>
       <c r="F31">
-        <v>167990</v>
+        <v>727600</v>
       </c>
       <c r="G31">
-        <v>197000</v>
+        <v>850000</v>
       </c>
       <c r="H31">
-        <v>354000</v>
+        <v>1690000</v>
       </c>
       <c r="I31">
-        <v>157000</v>
+        <v>840000</v>
       </c>
       <c r="J31" t="str">
-        <v>44.4%</v>
+        <v>49.7%</v>
       </c>
       <c r="K31">
-        <v>372000</v>
+        <v>1775000</v>
       </c>
       <c r="L31">
-        <v>18000</v>
+        <v>85000</v>
       </c>
       <c r="M31" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N31">
-        <v>447000</v>
+        <v>2130000</v>
       </c>
     </row>
     <row r="32">
@@ -3813,37 +3848,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E32" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F32">
-        <v>795408</v>
+        <v>167990</v>
       </c>
       <c r="G32">
-        <v>1020000</v>
+        <v>197000</v>
       </c>
       <c r="H32">
-        <v>1890000</v>
+        <v>354000</v>
       </c>
       <c r="I32">
-        <v>870000</v>
+        <v>157000</v>
       </c>
       <c r="J32" t="str">
-        <v>46.0%</v>
+        <v>44.4%</v>
       </c>
       <c r="K32">
-        <v>1985000</v>
+        <v>372000</v>
       </c>
       <c r="L32">
-        <v>95000</v>
+        <v>18000</v>
       </c>
       <c r="M32" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N32">
-        <v>2382000</v>
+        <v>447000</v>
       </c>
     </row>
     <row r="33">
@@ -3857,37 +3892,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E33" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F33">
-        <v>306020</v>
+        <v>795408</v>
       </c>
       <c r="G33">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="H33">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="I33">
-        <v>298000</v>
+        <v>870000</v>
       </c>
       <c r="J33" t="str">
-        <v>44.5%</v>
+        <v>46.0%</v>
       </c>
       <c r="K33">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
       <c r="L33">
-        <v>34000</v>
+        <v>95000</v>
       </c>
       <c r="M33" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N33">
-        <v>845000</v>
+        <v>2382000</v>
       </c>
     </row>
     <row r="34">
@@ -3901,37 +3936,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E34" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F34">
-        <v>668157</v>
+        <v>306020</v>
       </c>
       <c r="G34">
-        <v>780000</v>
+        <v>372000</v>
       </c>
       <c r="H34">
-        <v>1495000</v>
+        <v>670000</v>
       </c>
       <c r="I34">
-        <v>715000</v>
+        <v>298000</v>
       </c>
       <c r="J34" t="str">
-        <v>47.8%</v>
+        <v>44.5%</v>
       </c>
       <c r="K34">
-        <v>1570000</v>
+        <v>704000</v>
       </c>
       <c r="L34">
-        <v>75000</v>
+        <v>34000</v>
       </c>
       <c r="M34" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N34">
-        <v>1884000</v>
+        <v>845000</v>
       </c>
     </row>
     <row r="35">
@@ -3945,37 +3980,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E35" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F35">
-        <v>259549</v>
+        <v>668157</v>
       </c>
       <c r="G35">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="H35">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="I35">
-        <v>289000</v>
+        <v>715000</v>
       </c>
       <c r="J35" t="str">
-        <v>48.2%</v>
+        <v>47.8%</v>
       </c>
       <c r="K35">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
       <c r="L35">
-        <v>30000</v>
+        <v>75000</v>
       </c>
       <c r="M35" t="str">
         <v>5.0%</v>
       </c>
       <c r="N35">
-        <v>755000</v>
+        <v>1884000</v>
       </c>
     </row>
     <row r="36">
@@ -3989,37 +4024,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E36" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F36">
-        <v>828486</v>
+        <v>259549</v>
       </c>
       <c r="G36">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="H36">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="I36">
-        <v>880000</v>
+        <v>289000</v>
       </c>
       <c r="J36" t="str">
-        <v>46.8%</v>
+        <v>48.2%</v>
       </c>
       <c r="K36">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
       <c r="L36">
-        <v>94000</v>
+        <v>30000</v>
       </c>
       <c r="M36" t="str">
         <v>5.0%</v>
       </c>
       <c r="N36">
-        <v>2369000</v>
+        <v>755000</v>
       </c>
     </row>
     <row r="37">
@@ -4033,37 +4068,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F37">
-        <v>672571</v>
+        <v>828486</v>
       </c>
       <c r="G37">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H37">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="I37">
-        <v>690000</v>
+        <v>880000</v>
       </c>
       <c r="J37" t="str">
-        <v>46.3%</v>
+        <v>46.8%</v>
       </c>
       <c r="K37">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
       <c r="L37">
-        <v>75000</v>
+        <v>94000</v>
       </c>
       <c r="M37" t="str">
         <v>5.0%</v>
       </c>
       <c r="N37">
-        <v>1878000</v>
+        <v>2369000</v>
       </c>
     </row>
     <row r="38">
@@ -4077,37 +4112,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F38">
-        <v>399987</v>
+        <v>672571</v>
       </c>
       <c r="G38">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="H38">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="I38">
-        <v>440000</v>
+        <v>690000</v>
       </c>
       <c r="J38" t="str">
         <v>46.3%</v>
       </c>
       <c r="K38">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
       <c r="L38">
-        <v>48000</v>
+        <v>75000</v>
       </c>
       <c r="M38" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N38">
-        <v>1198000</v>
+        <v>1878000</v>
       </c>
     </row>
     <row r="39">
@@ -4121,13 +4156,13 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F39">
-        <v>389541</v>
+        <v>399987</v>
       </c>
       <c r="G39">
         <v>510000</v>
@@ -4165,37 +4200,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E40" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F40">
-        <v>468762</v>
+        <v>389541</v>
       </c>
       <c r="G40">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="H40">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="I40">
-        <v>590000</v>
+        <v>440000</v>
       </c>
       <c r="J40" t="str">
-        <v>49.6%</v>
+        <v>46.3%</v>
       </c>
       <c r="K40">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
       <c r="L40">
-        <v>60000</v>
+        <v>48000</v>
       </c>
       <c r="M40" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N40">
-        <v>1500000</v>
+        <v>1198000</v>
       </c>
     </row>
     <row r="41">
@@ -4209,37 +4244,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E41" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F41">
-        <v>200752</v>
+        <v>468762</v>
       </c>
       <c r="G41">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="H41">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="I41">
-        <v>230000</v>
+        <v>590000</v>
       </c>
       <c r="J41" t="str">
-        <v>46.9%</v>
+        <v>49.6%</v>
       </c>
       <c r="K41">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
       <c r="L41">
-        <v>25000</v>
+        <v>60000</v>
       </c>
       <c r="M41" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N41">
-        <v>618000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="42">
@@ -4253,37 +4288,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F42">
-        <v>550047</v>
+        <v>200752</v>
       </c>
       <c r="G42">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="H42">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="I42">
-        <v>605000</v>
+        <v>230000</v>
       </c>
       <c r="J42" t="str">
         <v>46.9%</v>
       </c>
       <c r="K42">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
       <c r="L42">
-        <v>65000</v>
+        <v>25000</v>
       </c>
       <c r="M42" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N42">
-        <v>1626000</v>
+        <v>618000</v>
       </c>
     </row>
     <row r="43">
@@ -4297,37 +4332,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E43" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F43">
-        <v>545604</v>
+        <v>550047</v>
       </c>
       <c r="G43">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="H43">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="I43">
-        <v>530000</v>
+        <v>605000</v>
       </c>
       <c r="J43" t="str">
-        <v>44.5%</v>
+        <v>46.9%</v>
       </c>
       <c r="K43">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
       <c r="L43">
-        <v>60000</v>
+        <v>65000</v>
       </c>
       <c r="M43" t="str">
         <v>5.0%</v>
       </c>
       <c r="N43">
-        <v>1500000</v>
+        <v>1626000</v>
       </c>
     </row>
     <row r="44">
@@ -4341,37 +4376,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E44" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F44">
-        <v>936250</v>
+        <v>545604</v>
       </c>
       <c r="G44">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="H44">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="I44">
-        <v>1060000</v>
+        <v>530000</v>
       </c>
       <c r="J44" t="str">
-        <v>48.4%</v>
+        <v>44.5%</v>
       </c>
       <c r="K44">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
       <c r="L44">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="M44" t="str">
         <v>5.0%</v>
       </c>
       <c r="N44">
-        <v>2760000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="45">
@@ -4379,43 +4414,43 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C45" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E45" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F45">
-        <v>203634</v>
+        <v>936250</v>
       </c>
       <c r="G45">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="H45">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="I45">
-        <v>202000</v>
+        <v>1060000</v>
       </c>
       <c r="J45" t="str">
-        <v>43.3%</v>
+        <v>48.4%</v>
       </c>
       <c r="K45">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
       <c r="L45">
-        <v>24000</v>
+        <v>110000</v>
       </c>
       <c r="M45" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N45">
-        <v>590000</v>
+        <v>2760000</v>
       </c>
     </row>
     <row r="46">
@@ -4429,37 +4464,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2662</v>
+        <v>TK-2201</v>
       </c>
       <c r="E46" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F46">
-        <v>238375</v>
+        <v>203634</v>
       </c>
       <c r="G46">
-        <v>320000</v>
+        <v>265000</v>
       </c>
       <c r="H46">
-        <v>590000</v>
+        <v>467000</v>
       </c>
       <c r="I46">
-        <v>270000</v>
+        <v>202000</v>
       </c>
       <c r="J46" t="str">
-        <v>45.8%</v>
+        <v>43.3%</v>
       </c>
       <c r="K46">
-        <v>620000</v>
+        <v>491000</v>
       </c>
       <c r="L46">
-        <v>30000</v>
+        <v>24000</v>
       </c>
       <c r="M46" t="str">
         <v>5.1%</v>
       </c>
       <c r="N46">
-        <v>744000</v>
+        <v>590000</v>
       </c>
     </row>
     <row r="47">
@@ -4473,37 +4508,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2882C</v>
+        <v>TK-2662</v>
       </c>
       <c r="E47" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F47">
-        <v>266199</v>
+        <v>238375</v>
       </c>
       <c r="G47">
-        <v>351000</v>
+        <v>320000</v>
       </c>
       <c r="H47">
-        <v>630000</v>
+        <v>590000</v>
       </c>
       <c r="I47">
-        <v>279000</v>
+        <v>270000</v>
       </c>
       <c r="J47" t="str">
-        <v>44.3%</v>
+        <v>45.8%</v>
       </c>
       <c r="K47">
-        <v>662000</v>
+        <v>620000</v>
       </c>
       <c r="L47">
-        <v>32000</v>
+        <v>30000</v>
       </c>
       <c r="M47" t="str">
         <v>5.1%</v>
       </c>
       <c r="N47">
-        <v>795000</v>
+        <v>744000</v>
       </c>
     </row>
     <row r="48">
@@ -4517,37 +4552,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-3030C</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F48">
-        <v>290175</v>
+        <v>266199</v>
       </c>
       <c r="G48">
-        <v>375000</v>
+        <v>351000</v>
       </c>
       <c r="H48">
-        <v>750000</v>
+        <v>630000</v>
       </c>
       <c r="I48">
-        <v>375000</v>
+        <v>279000</v>
       </c>
       <c r="J48" t="str">
-        <v>50.0%</v>
+        <v>44.3%</v>
       </c>
       <c r="K48">
-        <v>788000</v>
+        <v>662000</v>
       </c>
       <c r="L48">
-        <v>38000</v>
+        <v>32000</v>
       </c>
       <c r="M48" t="str">
         <v>5.1%</v>
       </c>
       <c r="N48">
-        <v>946000</v>
+        <v>795000</v>
       </c>
     </row>
     <row r="49">
@@ -4558,40 +4593,40 @@
         <v>Takin</v>
       </c>
       <c r="C49" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-036A</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E49" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F49">
-        <v>433985</v>
+        <v>290175</v>
       </c>
       <c r="G49">
-        <v>515000</v>
+        <v>375000</v>
       </c>
       <c r="H49">
-        <v>891000</v>
+        <v>750000</v>
       </c>
       <c r="I49">
-        <v>376000</v>
+        <v>375000</v>
       </c>
       <c r="J49" t="str">
-        <v>42.2%</v>
+        <v>50.0%</v>
       </c>
       <c r="K49">
-        <v>936000</v>
+        <v>788000</v>
       </c>
       <c r="L49">
-        <v>45000</v>
+        <v>38000</v>
       </c>
       <c r="M49" t="str">
         <v>5.1%</v>
       </c>
       <c r="N49">
-        <v>1124000</v>
+        <v>946000</v>
       </c>
     </row>
     <row r="50">
@@ -4605,37 +4640,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-0324</v>
+        <v>TK-036A</v>
       </c>
       <c r="E50" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F50">
-        <v>188524</v>
+        <v>433985</v>
       </c>
       <c r="G50">
-        <v>245000</v>
+        <v>515000</v>
       </c>
       <c r="H50">
-        <v>441000</v>
+        <v>891000</v>
       </c>
       <c r="I50">
-        <v>196000</v>
+        <v>376000</v>
       </c>
       <c r="J50" t="str">
-        <v>44.4%</v>
+        <v>42.2%</v>
       </c>
       <c r="K50">
-        <v>464000</v>
+        <v>936000</v>
       </c>
       <c r="L50">
-        <v>23000</v>
+        <v>45000</v>
       </c>
       <c r="M50" t="str">
-        <v>5.2%</v>
+        <v>5.1%</v>
       </c>
       <c r="N50">
-        <v>557000</v>
+        <v>1124000</v>
       </c>
     </row>
     <row r="51">
@@ -4649,37 +4684,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0348A</v>
+        <v>TK-0324</v>
       </c>
       <c r="E51" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F51">
-        <v>492000</v>
+        <v>188524</v>
       </c>
       <c r="G51">
-        <v>580000</v>
+        <v>245000</v>
       </c>
       <c r="H51">
-        <v>1044000</v>
+        <v>441000</v>
       </c>
       <c r="I51">
-        <v>464000</v>
+        <v>196000</v>
       </c>
       <c r="J51" t="str">
         <v>44.4%</v>
       </c>
       <c r="K51">
-        <v>1097000</v>
+        <v>464000</v>
       </c>
       <c r="L51">
-        <v>53000</v>
+        <v>23000</v>
       </c>
       <c r="M51" t="str">
-        <v>5.1%</v>
+        <v>5.2%</v>
       </c>
       <c r="N51">
-        <v>1317000</v>
+        <v>557000</v>
       </c>
     </row>
     <row r="52">
@@ -4693,37 +4728,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0369</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F52">
-        <v>419848</v>
+        <v>492000</v>
       </c>
       <c r="G52">
-        <v>535000</v>
+        <v>580000</v>
       </c>
       <c r="H52">
-        <v>969000</v>
+        <v>1044000</v>
       </c>
       <c r="I52">
-        <v>434000</v>
+        <v>464000</v>
       </c>
       <c r="J52" t="str">
-        <v>44.8%</v>
+        <v>44.4%</v>
       </c>
       <c r="K52">
-        <v>1018000</v>
+        <v>1097000</v>
       </c>
       <c r="L52">
-        <v>49000</v>
+        <v>53000</v>
       </c>
       <c r="M52" t="str">
         <v>5.1%</v>
       </c>
       <c r="N52">
-        <v>1222000</v>
+        <v>1317000</v>
       </c>
     </row>
     <row r="53">
@@ -4737,37 +4772,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0488</v>
+        <v>TK-0369</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F53">
-        <v>672571</v>
+        <v>419848</v>
       </c>
       <c r="G53">
-        <v>810000</v>
+        <v>535000</v>
       </c>
       <c r="H53">
-        <v>1469000</v>
+        <v>969000</v>
       </c>
       <c r="I53">
-        <v>659000</v>
+        <v>434000</v>
       </c>
       <c r="J53" t="str">
-        <v>44.9%</v>
+        <v>44.8%</v>
       </c>
       <c r="K53">
-        <v>1543000</v>
+        <v>1018000</v>
       </c>
       <c r="L53">
-        <v>74000</v>
+        <v>49000</v>
       </c>
       <c r="M53" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N53">
-        <v>1852000</v>
+        <v>1222000</v>
       </c>
     </row>
     <row r="54">
@@ -4778,40 +4813,40 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-468</v>
+        <v>TK-0488</v>
       </c>
       <c r="E54" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F54">
-        <v>366857</v>
+        <v>672571</v>
       </c>
       <c r="G54">
-        <v>452000</v>
+        <v>810000</v>
       </c>
       <c r="H54">
-        <v>900000</v>
+        <v>1469000</v>
       </c>
       <c r="I54">
-        <v>448000</v>
+        <v>659000</v>
       </c>
       <c r="J54" t="str">
-        <v>49.8%</v>
+        <v>44.9%</v>
       </c>
       <c r="K54">
-        <v>945000</v>
+        <v>1543000</v>
       </c>
       <c r="L54">
-        <v>45000</v>
+        <v>74000</v>
       </c>
       <c r="M54" t="str">
         <v>5.0%</v>
       </c>
       <c r="N54">
-        <v>1134000</v>
+        <v>1852000</v>
       </c>
     </row>
     <row r="55">
@@ -4825,37 +4860,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-469</v>
+        <v>TK-468</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F55">
-        <v>468762</v>
+        <v>366857</v>
       </c>
       <c r="G55">
-        <v>615000</v>
+        <v>452000</v>
       </c>
       <c r="H55">
-        <v>1050000</v>
+        <v>900000</v>
       </c>
       <c r="I55">
-        <v>435000</v>
+        <v>448000</v>
       </c>
       <c r="J55" t="str">
-        <v>41.4%</v>
+        <v>49.8%</v>
       </c>
       <c r="K55">
-        <v>1103000</v>
+        <v>945000</v>
       </c>
       <c r="L55">
-        <v>53000</v>
+        <v>45000</v>
       </c>
       <c r="M55" t="str">
         <v>5.0%</v>
       </c>
       <c r="N55">
-        <v>1324000</v>
+        <v>1134000</v>
       </c>
     </row>
     <row r="56">
@@ -4869,37 +4904,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-1002</v>
+        <v>TK-469</v>
       </c>
       <c r="E56" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F56">
-        <v>128400</v>
+        <v>468762</v>
       </c>
       <c r="G56">
-        <v>158000</v>
+        <v>615000</v>
       </c>
       <c r="H56">
-        <v>270000</v>
+        <v>1050000</v>
       </c>
       <c r="I56">
-        <v>112000</v>
+        <v>435000</v>
       </c>
       <c r="J56" t="str">
-        <v>41.5%</v>
+        <v>41.4%</v>
       </c>
       <c r="K56">
-        <v>284000</v>
+        <v>1103000</v>
       </c>
       <c r="L56">
-        <v>14000</v>
+        <v>53000</v>
       </c>
       <c r="M56" t="str">
-        <v>5.2%</v>
+        <v>5.0%</v>
       </c>
       <c r="N56">
-        <v>341000</v>
+        <v>1324000</v>
       </c>
     </row>
     <row r="57">
@@ -4913,49 +4948,93 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1003</v>
+        <v>TK-1002</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 3 bóng Takin</v>
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
       </c>
       <c r="F57">
-        <v>157290</v>
+        <v>128400</v>
       </c>
       <c r="G57">
-        <v>194000</v>
+        <v>158000</v>
       </c>
       <c r="H57">
-        <v>330000</v>
+        <v>270000</v>
       </c>
       <c r="I57">
-        <v>136000</v>
+        <v>112000</v>
       </c>
       <c r="J57" t="str">
-        <v>41.2%</v>
+        <v>41.5%</v>
       </c>
       <c r="K57">
-        <v>347000</v>
+        <v>284000</v>
       </c>
       <c r="L57">
-        <v>17000</v>
+        <v>14000</v>
       </c>
       <c r="M57" t="str">
         <v>5.2%</v>
       </c>
       <c r="N57">
+        <v>341000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C58" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D58" t="str">
+        <v>TK-1003</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
+      </c>
+      <c r="F58">
+        <v>157290</v>
+      </c>
+      <c r="G58">
+        <v>194000</v>
+      </c>
+      <c r="H58">
+        <v>330000</v>
+      </c>
+      <c r="I58">
+        <v>136000</v>
+      </c>
+      <c r="J58" t="str">
+        <v>41.2%</v>
+      </c>
+      <c r="K58">
+        <v>347000</v>
+      </c>
+      <c r="L58">
+        <v>17000</v>
+      </c>
+      <c r="M58" t="str">
+        <v>5.2%</v>
+      </c>
+      <c r="N58">
         <v>417000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N58"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -5742,31 +5821,31 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D21" t="str">
-        <v>LK-3386A</v>
+        <v>LK-3348</v>
       </c>
       <c r="E21" t="str">
-        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+        <v>Bộ nồi Táo Lock&amp;king 3 món inox cao cấp</v>
       </c>
       <c r="F21">
-        <v>530000</v>
+        <v>580000</v>
       </c>
       <c r="G21">
-        <v>550000</v>
+        <v>580000</v>
       </c>
       <c r="H21">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I21" t="str">
-        <v>3.8%</v>
+        <v>0.0%</v>
       </c>
       <c r="J21" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K21">
-        <v>990000</v>
+        <v>1044000</v>
       </c>
       <c r="L21">
-        <v>1040000</v>
+        <v>1097000</v>
       </c>
     </row>
     <row r="22">
@@ -5780,31 +5859,31 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D22" t="str">
-        <v>LK-3568A</v>
+        <v>LK-3386A</v>
       </c>
       <c r="E22" t="str">
-        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
       </c>
       <c r="F22">
-        <v>940000</v>
+        <v>530000</v>
       </c>
       <c r="G22">
-        <v>960000</v>
+        <v>550000</v>
       </c>
       <c r="H22">
         <v>20000</v>
       </c>
       <c r="I22" t="str">
-        <v>2.1%</v>
+        <v>3.8%</v>
       </c>
       <c r="J22" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K22">
-        <v>1690000</v>
+        <v>990000</v>
       </c>
       <c r="L22">
-        <v>1775000</v>
+        <v>1040000</v>
       </c>
     </row>
     <row r="23">
@@ -5815,34 +5894,34 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C23" t="str">
-        <v>NỒI TĂNG ÁP</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D23" t="str">
-        <v>LK-3122</v>
+        <v>LK-3568A</v>
       </c>
       <c r="E23" t="str">
-        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
       </c>
       <c r="F23">
-        <v>460000</v>
+        <v>940000</v>
       </c>
       <c r="G23">
-        <v>470000</v>
+        <v>960000</v>
       </c>
       <c r="H23">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="I23" t="str">
-        <v>2.2%</v>
+        <v>2.1%</v>
       </c>
       <c r="J23" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K23">
-        <v>820000</v>
+        <v>1690000</v>
       </c>
       <c r="L23">
-        <v>886000</v>
+        <v>1775000</v>
       </c>
     </row>
     <row r="24">
@@ -5856,31 +5935,31 @@
         <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D24" t="str">
-        <v>LK-3126</v>
+        <v>LK-3122</v>
       </c>
       <c r="E24" t="str">
-        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
       </c>
       <c r="F24">
-        <v>525000</v>
+        <v>460000</v>
       </c>
       <c r="G24">
-        <v>535000</v>
+        <v>470000</v>
       </c>
       <c r="H24">
         <v>10000</v>
       </c>
       <c r="I24" t="str">
-        <v>1.9%</v>
+        <v>2.2%</v>
       </c>
       <c r="J24" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K24">
-        <v>990000</v>
+        <v>820000</v>
       </c>
       <c r="L24">
-        <v>1070000</v>
+        <v>886000</v>
       </c>
     </row>
     <row r="25">
@@ -5891,34 +5970,34 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C25" t="str">
-        <v>ẤM &amp; BÌNH</v>
+        <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D25" t="str">
-        <v>LK-1038</v>
+        <v>LK-3126</v>
       </c>
       <c r="E25" t="str">
-        <v>Ấm đun nước LK-1038</v>
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
       </c>
       <c r="F25">
-        <v>300000</v>
+        <v>525000</v>
       </c>
       <c r="G25">
-        <v>300000</v>
+        <v>535000</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I25" t="str">
-        <v>0.0%</v>
+        <v>1.9%</v>
       </c>
       <c r="J25" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K25">
-        <v>525000</v>
+        <v>990000</v>
       </c>
       <c r="L25">
-        <v>552000</v>
+        <v>1070000</v>
       </c>
     </row>
     <row r="26">
@@ -5929,19 +6008,19 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C26" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>ẤM &amp; BÌNH</v>
       </c>
       <c r="D26" t="str">
-        <v>LK-92</v>
+        <v>LK-1038</v>
       </c>
       <c r="E26" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Ấm đun nước LK-1038</v>
       </c>
       <c r="F26">
-        <v>835000</v>
+        <v>300000</v>
       </c>
       <c r="G26">
-        <v>835000</v>
+        <v>300000</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -5953,10 +6032,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K26">
-        <v>1590000</v>
+        <v>525000</v>
       </c>
       <c r="L26">
-        <v>1670000</v>
+        <v>552000</v>
       </c>
     </row>
     <row r="27">
@@ -5970,16 +6049,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D27" t="str">
-        <v>LK-586</v>
+        <v>LK-92</v>
       </c>
       <c r="E27" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F27">
-        <v>430000</v>
+        <v>835000</v>
       </c>
       <c r="G27">
-        <v>430000</v>
+        <v>835000</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -5991,10 +6070,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K27">
-        <v>745000</v>
+        <v>1590000</v>
       </c>
       <c r="L27">
-        <v>783000</v>
+        <v>1670000</v>
       </c>
     </row>
     <row r="28">
@@ -6008,16 +6087,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D28" t="str">
-        <v>LK-588</v>
+        <v>LK-586</v>
       </c>
       <c r="E28" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F28">
-        <v>585000</v>
+        <v>430000</v>
       </c>
       <c r="G28">
-        <v>585000</v>
+        <v>430000</v>
       </c>
       <c r="H28">
         <v>0</v>
@@ -6029,10 +6108,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K28">
-        <v>1050000</v>
+        <v>745000</v>
       </c>
       <c r="L28">
-        <v>1103000</v>
+        <v>783000</v>
       </c>
     </row>
     <row r="29">
@@ -6046,16 +6125,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D29" t="str">
-        <v>LK-668</v>
+        <v>LK-588</v>
       </c>
       <c r="E29" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F29">
-        <v>460000</v>
+        <v>585000</v>
       </c>
       <c r="G29">
-        <v>460000</v>
+        <v>585000</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -6067,10 +6146,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K29">
-        <v>920000</v>
+        <v>1050000</v>
       </c>
       <c r="L29">
-        <v>966000</v>
+        <v>1103000</v>
       </c>
     </row>
     <row r="30">
@@ -6084,16 +6163,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D30" t="str">
-        <v>LK-688</v>
+        <v>LK-668</v>
       </c>
       <c r="E30" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
       </c>
       <c r="F30">
-        <v>850000</v>
+        <v>460000</v>
       </c>
       <c r="G30">
-        <v>850000</v>
+        <v>460000</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -6105,10 +6184,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K30">
-        <v>1690000</v>
+        <v>920000</v>
       </c>
       <c r="L30">
-        <v>1775000</v>
+        <v>966000</v>
       </c>
     </row>
     <row r="31">
@@ -6122,16 +6201,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D31" t="str">
-        <v>LK-1003</v>
+        <v>LK-688</v>
       </c>
       <c r="E31" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
       </c>
       <c r="F31">
-        <v>197000</v>
+        <v>850000</v>
       </c>
       <c r="G31">
-        <v>197000</v>
+        <v>850000</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -6143,10 +6222,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K31">
-        <v>354000</v>
+        <v>1690000</v>
       </c>
       <c r="L31">
-        <v>372000</v>
+        <v>1775000</v>
       </c>
     </row>
     <row r="32">
@@ -6160,16 +6239,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E32" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F32">
-        <v>1020000</v>
+        <v>197000</v>
       </c>
       <c r="G32">
-        <v>1020000</v>
+        <v>197000</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -6181,10 +6260,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K32">
-        <v>1890000</v>
+        <v>354000</v>
       </c>
       <c r="L32">
-        <v>1985000</v>
+        <v>372000</v>
       </c>
     </row>
     <row r="33">
@@ -6198,16 +6277,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E33" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F33">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="G33">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="H33">
         <v>0</v>
@@ -6219,10 +6298,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K33">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="L33">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
     </row>
     <row r="34">
@@ -6236,31 +6315,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E34" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F34">
-        <v>890000</v>
+        <v>372000</v>
       </c>
       <c r="G34">
-        <v>780000</v>
+        <v>372000</v>
       </c>
       <c r="H34">
-        <v>-110000</v>
+        <v>0</v>
       </c>
       <c r="I34" t="str">
-        <v>-12.4%</v>
+        <v>0.0%</v>
       </c>
       <c r="J34" t="str">
-        <v>Giảm giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K34">
-        <v>1495000</v>
+        <v>670000</v>
       </c>
       <c r="L34">
-        <v>1570000</v>
+        <v>704000</v>
       </c>
     </row>
     <row r="35">
@@ -6274,31 +6353,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E35" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F35">
-        <v>340000</v>
+        <v>890000</v>
       </c>
       <c r="G35">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="H35">
-        <v>-30000</v>
+        <v>-110000</v>
       </c>
       <c r="I35" t="str">
-        <v>-8.8%</v>
+        <v>-12.4%</v>
       </c>
       <c r="J35" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K35">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="L35">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
     </row>
     <row r="36">
@@ -6312,31 +6391,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E36" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F36">
-        <v>1080000</v>
+        <v>340000</v>
       </c>
       <c r="G36">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="H36">
-        <v>-80000</v>
+        <v>-30000</v>
       </c>
       <c r="I36" t="str">
-        <v>-7.4%</v>
+        <v>-8.8%</v>
       </c>
       <c r="J36" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K36">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="L36">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
     </row>
     <row r="37">
@@ -6350,31 +6429,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F37">
-        <v>850000</v>
+        <v>1080000</v>
       </c>
       <c r="G37">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H37">
-        <v>-50000</v>
+        <v>-80000</v>
       </c>
       <c r="I37" t="str">
-        <v>-5.9%</v>
+        <v>-7.4%</v>
       </c>
       <c r="J37" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K37">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="L37">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
     </row>
     <row r="38">
@@ -6388,31 +6467,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F38">
-        <v>510000</v>
+        <v>850000</v>
       </c>
       <c r="G38">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="I38" t="str">
-        <v>0.0%</v>
+        <v>-5.9%</v>
       </c>
       <c r="J38" t="str">
-        <v>Giữ nguyên</v>
+        <v>Giảm giá</v>
       </c>
       <c r="K38">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="L38">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
     </row>
     <row r="39">
@@ -6426,10 +6505,10 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F39">
         <v>510000</v>
@@ -6464,16 +6543,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E40" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F40">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="G40">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -6485,10 +6564,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K40">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="L40">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
     </row>
     <row r="41">
@@ -6502,16 +6581,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E41" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F41">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="G41">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="H41">
         <v>0</v>
@@ -6523,10 +6602,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K41">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="L41">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
     </row>
     <row r="42">
@@ -6540,16 +6619,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F42">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="G42">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="H42">
         <v>0</v>
@@ -6561,10 +6640,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K42">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="L42">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
     </row>
     <row r="43">
@@ -6578,31 +6657,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E43" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F43">
-        <v>710000</v>
+        <v>685000</v>
       </c>
       <c r="G43">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="H43">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="I43" t="str">
-        <v>-7.0%</v>
+        <v>0.0%</v>
       </c>
       <c r="J43" t="str">
-        <v>Giảm giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K43">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="L43">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
     </row>
     <row r="44">
@@ -6616,31 +6695,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E44" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F44">
-        <v>1130000</v>
+        <v>710000</v>
       </c>
       <c r="G44">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="I44" t="str">
-        <v>0.0%</v>
+        <v>-7.0%</v>
       </c>
       <c r="J44" t="str">
-        <v>Giữ nguyên</v>
+        <v>Giảm giá</v>
       </c>
       <c r="K44">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="L44">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
     </row>
     <row r="45">
@@ -6648,37 +6727,37 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C45" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E45" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F45">
-        <v>260000</v>
+        <v>1130000</v>
       </c>
       <c r="G45">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="H45">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="I45" t="str">
-        <v>1.9%</v>
+        <v>0.0%</v>
       </c>
       <c r="J45" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K45">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="L45">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
     </row>
     <row r="46">
@@ -6692,31 +6771,31 @@
         <v>CHẢO</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2662</v>
+        <v>TK-2201</v>
       </c>
       <c r="E46" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F46">
-        <v>310000</v>
+        <v>260000</v>
       </c>
       <c r="G46">
-        <v>320000</v>
+        <v>265000</v>
       </c>
       <c r="H46">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="I46" t="str">
-        <v>3.2%</v>
+        <v>1.9%</v>
       </c>
       <c r="J46" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K46">
-        <v>590000</v>
+        <v>467000</v>
       </c>
       <c r="L46">
-        <v>620000</v>
+        <v>491000</v>
       </c>
     </row>
     <row r="47">
@@ -6730,31 +6809,31 @@
         <v>CHẢO</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2882C</v>
+        <v>TK-2662</v>
       </c>
       <c r="E47" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F47">
-        <v>341000</v>
+        <v>310000</v>
       </c>
       <c r="G47">
-        <v>351000</v>
+        <v>320000</v>
       </c>
       <c r="H47">
         <v>10000</v>
       </c>
       <c r="I47" t="str">
-        <v>2.9%</v>
+        <v>3.2%</v>
       </c>
       <c r="J47" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K47">
-        <v>630000</v>
+        <v>590000</v>
       </c>
       <c r="L47">
-        <v>662000</v>
+        <v>620000</v>
       </c>
     </row>
     <row r="48">
@@ -6768,31 +6847,31 @@
         <v>CHẢO</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-3030C</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F48">
-        <v>360000</v>
+        <v>341000</v>
       </c>
       <c r="G48">
-        <v>375000</v>
+        <v>351000</v>
       </c>
       <c r="H48">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="I48" t="str">
-        <v>4.2%</v>
+        <v>2.9%</v>
       </c>
       <c r="J48" t="str">
         <v>Tăng giá</v>
       </c>
       <c r="K48">
-        <v>750000</v>
+        <v>630000</v>
       </c>
       <c r="L48">
-        <v>788000</v>
+        <v>662000</v>
       </c>
     </row>
     <row r="49">
@@ -6803,34 +6882,34 @@
         <v>Takin</v>
       </c>
       <c r="C49" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-036A</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E49" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F49">
-        <v>515000</v>
+        <v>360000</v>
       </c>
       <c r="G49">
-        <v>515000</v>
+        <v>375000</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I49" t="str">
-        <v>0.0%</v>
+        <v>4.2%</v>
       </c>
       <c r="J49" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K49">
-        <v>891000</v>
+        <v>750000</v>
       </c>
       <c r="L49">
-        <v>936000</v>
+        <v>788000</v>
       </c>
     </row>
     <row r="50">
@@ -6844,16 +6923,16 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-0324</v>
+        <v>TK-036A</v>
       </c>
       <c r="E50" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F50">
-        <v>245000</v>
+        <v>515000</v>
       </c>
       <c r="G50">
-        <v>245000</v>
+        <v>515000</v>
       </c>
       <c r="H50">
         <v>0</v>
@@ -6865,10 +6944,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K50">
-        <v>441000</v>
+        <v>891000</v>
       </c>
       <c r="L50">
-        <v>464000</v>
+        <v>936000</v>
       </c>
     </row>
     <row r="51">
@@ -6882,16 +6961,16 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0348A</v>
+        <v>TK-0324</v>
       </c>
       <c r="E51" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F51">
-        <v>580000</v>
+        <v>245000</v>
       </c>
       <c r="G51">
-        <v>580000</v>
+        <v>245000</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -6903,10 +6982,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K51">
-        <v>1044000</v>
+        <v>441000</v>
       </c>
       <c r="L51">
-        <v>1097000</v>
+        <v>464000</v>
       </c>
     </row>
     <row r="52">
@@ -6920,16 +6999,16 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0369</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F52">
-        <v>535000</v>
+        <v>580000</v>
       </c>
       <c r="G52">
-        <v>535000</v>
+        <v>580000</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -6941,10 +7020,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K52">
-        <v>969000</v>
+        <v>1044000</v>
       </c>
       <c r="L52">
-        <v>1018000</v>
+        <v>1097000</v>
       </c>
     </row>
     <row r="53">
@@ -6958,16 +7037,16 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0488</v>
+        <v>TK-0369</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F53">
-        <v>810000</v>
+        <v>535000</v>
       </c>
       <c r="G53">
-        <v>810000</v>
+        <v>535000</v>
       </c>
       <c r="H53">
         <v>0</v>
@@ -6979,10 +7058,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K53">
-        <v>1469000</v>
+        <v>969000</v>
       </c>
       <c r="L53">
-        <v>1543000</v>
+        <v>1018000</v>
       </c>
     </row>
     <row r="54">
@@ -6993,19 +7072,19 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-468</v>
+        <v>TK-0488</v>
       </c>
       <c r="E54" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F54">
-        <v>452000</v>
+        <v>810000</v>
       </c>
       <c r="G54">
-        <v>452000</v>
+        <v>810000</v>
       </c>
       <c r="H54">
         <v>0</v>
@@ -7017,10 +7096,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K54">
-        <v>900000</v>
+        <v>1469000</v>
       </c>
       <c r="L54">
-        <v>945000</v>
+        <v>1543000</v>
       </c>
     </row>
     <row r="55">
@@ -7034,16 +7113,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-469</v>
+        <v>TK-468</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F55">
-        <v>615000</v>
+        <v>452000</v>
       </c>
       <c r="G55">
-        <v>615000</v>
+        <v>452000</v>
       </c>
       <c r="H55">
         <v>0</v>
@@ -7055,10 +7134,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K55">
-        <v>1050000</v>
+        <v>900000</v>
       </c>
       <c r="L55">
-        <v>1103000</v>
+        <v>945000</v>
       </c>
     </row>
     <row r="56">
@@ -7072,16 +7151,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-1002</v>
+        <v>TK-469</v>
       </c>
       <c r="E56" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F56">
-        <v>158000</v>
+        <v>615000</v>
       </c>
       <c r="G56">
-        <v>158000</v>
+        <v>615000</v>
       </c>
       <c r="H56">
         <v>0</v>
@@ -7093,10 +7172,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K56">
-        <v>270000</v>
+        <v>1050000</v>
       </c>
       <c r="L56">
-        <v>284000</v>
+        <v>1103000</v>
       </c>
     </row>
     <row r="57">
@@ -7110,16 +7189,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1003</v>
+        <v>TK-1002</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 3 bóng Takin</v>
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
       </c>
       <c r="F57">
-        <v>194000</v>
+        <v>158000</v>
       </c>
       <c r="G57">
-        <v>194000</v>
+        <v>158000</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -7131,15 +7210,53 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K57">
+        <v>270000</v>
+      </c>
+      <c r="L57">
+        <v>284000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C58" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D58" t="str">
+        <v>TK-1003</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
+      </c>
+      <c r="F58">
+        <v>194000</v>
+      </c>
+      <c r="G58">
+        <v>194000</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K58">
         <v>330000</v>
       </c>
-      <c r="L57">
+      <c r="L58">
         <v>347000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: them 6 san pham moi va cap nhat gia 2 san pham (quy mo toan he thong 63 model)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Bang_Gia_Chuan_57_Ma" sheetId="1" r:id="rId1"/>
+    <sheet name="Bang_Gia_Chuan_63_Ma" sheetId="1" r:id="rId1"/>
     <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
     <sheet name="BienDong_Gia_NPP" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K64"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1510,28 +1510,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1003</v>
+        <v>LK-6886</v>
       </c>
       <c r="E32" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo Model: LK 6886</v>
       </c>
       <c r="F32">
-        <v>197000</v>
+        <v>770000</v>
       </c>
       <c r="G32">
-        <v>354000</v>
+        <v>1490000</v>
       </c>
       <c r="H32">
-        <v>372000</v>
+        <v>1564500</v>
       </c>
       <c r="I32">
-        <v>447000</v>
+        <v>1878000</v>
       </c>
       <c r="J32">
-        <v>157000</v>
+        <v>720000</v>
       </c>
       <c r="K32" t="str">
-        <v>44.4%</v>
+        <v>48.3%</v>
       </c>
     </row>
     <row r="33">
@@ -1545,28 +1545,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E33" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F33">
-        <v>1020000</v>
+        <v>210000</v>
       </c>
       <c r="G33">
-        <v>1890000</v>
+        <v>399000</v>
       </c>
       <c r="H33">
-        <v>1985000</v>
+        <v>418950</v>
       </c>
       <c r="I33">
-        <v>2382000</v>
+        <v>503000</v>
       </c>
       <c r="J33">
-        <v>870000</v>
+        <v>189000</v>
       </c>
       <c r="K33" t="str">
-        <v>46.0%</v>
+        <v>47.4%</v>
       </c>
     </row>
     <row r="34">
@@ -1580,28 +1580,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E34" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F34">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="G34">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="H34">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
       <c r="I34">
-        <v>845000</v>
+        <v>2382000</v>
       </c>
       <c r="J34">
-        <v>298000</v>
+        <v>870000</v>
       </c>
       <c r="K34" t="str">
-        <v>44.5%</v>
+        <v>46.0%</v>
       </c>
     </row>
     <row r="35">
@@ -1615,28 +1615,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E35" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F35">
-        <v>780000</v>
+        <v>320000</v>
       </c>
       <c r="G35">
-        <v>1495000</v>
+        <v>620000</v>
       </c>
       <c r="H35">
-        <v>1570000</v>
+        <v>651000</v>
       </c>
       <c r="I35">
-        <v>1884000</v>
+        <v>782000</v>
       </c>
       <c r="J35">
-        <v>715000</v>
+        <v>300000</v>
       </c>
       <c r="K35" t="str">
-        <v>47.8%</v>
+        <v>48.4%</v>
       </c>
     </row>
     <row r="36">
@@ -1650,28 +1650,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E36" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F36">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="G36">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="H36">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
       <c r="I36">
-        <v>755000</v>
+        <v>1884000</v>
       </c>
       <c r="J36">
-        <v>289000</v>
+        <v>715000</v>
       </c>
       <c r="K36" t="str">
-        <v>48.2%</v>
+        <v>47.8%</v>
       </c>
     </row>
     <row r="37">
@@ -1685,28 +1685,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F37">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="G37">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="H37">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
       <c r="I37">
-        <v>2369000</v>
+        <v>755000</v>
       </c>
       <c r="J37">
-        <v>880000</v>
+        <v>289000</v>
       </c>
       <c r="K37" t="str">
-        <v>46.8%</v>
+        <v>48.2%</v>
       </c>
     </row>
     <row r="38">
@@ -1720,28 +1720,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F38">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="G38">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="H38">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
       <c r="I38">
-        <v>1878000</v>
+        <v>2369000</v>
       </c>
       <c r="J38">
-        <v>690000</v>
+        <v>880000</v>
       </c>
       <c r="K38" t="str">
-        <v>46.3%</v>
+        <v>46.8%</v>
       </c>
     </row>
     <row r="39">
@@ -1755,25 +1755,25 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F39">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="G39">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="H39">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
       <c r="I39">
-        <v>1198000</v>
+        <v>1878000</v>
       </c>
       <c r="J39">
-        <v>440000</v>
+        <v>690000</v>
       </c>
       <c r="K39" t="str">
         <v>46.3%</v>
@@ -1790,10 +1790,10 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E40" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F40">
         <v>510000</v>
@@ -1825,28 +1825,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E41" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F41">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="G41">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="H41">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
       <c r="I41">
-        <v>1500000</v>
+        <v>1198000</v>
       </c>
       <c r="J41">
-        <v>590000</v>
+        <v>440000</v>
       </c>
       <c r="K41" t="str">
-        <v>49.6%</v>
+        <v>46.3%</v>
       </c>
     </row>
     <row r="42">
@@ -1860,28 +1860,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F42">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="G42">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="H42">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
       <c r="I42">
-        <v>618000</v>
+        <v>1500000</v>
       </c>
       <c r="J42">
-        <v>230000</v>
+        <v>590000</v>
       </c>
       <c r="K42" t="str">
-        <v>46.9%</v>
+        <v>49.6%</v>
       </c>
     </row>
     <row r="43">
@@ -1895,25 +1895,25 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E43" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F43">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="G43">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="H43">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
       <c r="I43">
-        <v>1626000</v>
+        <v>618000</v>
       </c>
       <c r="J43">
-        <v>605000</v>
+        <v>230000</v>
       </c>
       <c r="K43" t="str">
         <v>46.9%</v>
@@ -1930,28 +1930,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E44" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F44">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="G44">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="H44">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
       <c r="I44">
-        <v>1500000</v>
+        <v>1626000</v>
       </c>
       <c r="J44">
-        <v>530000</v>
+        <v>605000</v>
       </c>
       <c r="K44" t="str">
-        <v>44.5%</v>
+        <v>46.9%</v>
       </c>
     </row>
     <row r="45">
@@ -1965,28 +1965,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E45" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F45">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="G45">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="H45">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
       <c r="I45">
-        <v>2760000</v>
+        <v>1500000</v>
       </c>
       <c r="J45">
-        <v>1060000</v>
+        <v>530000</v>
       </c>
       <c r="K45" t="str">
-        <v>48.4%</v>
+        <v>44.5%</v>
       </c>
     </row>
     <row r="46">
@@ -1994,34 +1994,34 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C46" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E46" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F46">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="G46">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="H46">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
       <c r="I46">
-        <v>590000</v>
+        <v>2760000</v>
       </c>
       <c r="J46">
-        <v>202000</v>
+        <v>1060000</v>
       </c>
       <c r="K46" t="str">
-        <v>43.3%</v>
+        <v>48.4%</v>
       </c>
     </row>
     <row r="47">
@@ -2029,34 +2029,34 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C47" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2662</v>
+        <v>LK-8989</v>
       </c>
       <c r="E47" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>Bếp từ đơn -2200W LK-8989</v>
       </c>
       <c r="F47">
-        <v>320000</v>
+        <v>790000</v>
       </c>
       <c r="G47">
-        <v>590000</v>
+        <v>1490000</v>
       </c>
       <c r="H47">
-        <v>620000</v>
+        <v>1564500</v>
       </c>
       <c r="I47">
-        <v>744000</v>
+        <v>1878000</v>
       </c>
       <c r="J47">
-        <v>270000</v>
+        <v>700000</v>
       </c>
       <c r="K47" t="str">
-        <v>45.8%</v>
+        <v>47.0%</v>
       </c>
     </row>
     <row r="48">
@@ -2064,34 +2064,34 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C48" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-2882C</v>
+        <v>LK-8924</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn -2400W LK-8924</v>
       </c>
       <c r="F48">
-        <v>351000</v>
+        <v>850000</v>
       </c>
       <c r="G48">
-        <v>630000</v>
+        <v>1590000</v>
       </c>
       <c r="H48">
-        <v>662000</v>
+        <v>1669500</v>
       </c>
       <c r="I48">
-        <v>795000</v>
+        <v>2004000</v>
       </c>
       <c r="J48">
-        <v>279000</v>
+        <v>740000</v>
       </c>
       <c r="K48" t="str">
-        <v>44.3%</v>
+        <v>46.5%</v>
       </c>
     </row>
     <row r="49">
@@ -2099,34 +2099,34 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C49" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-3030C</v>
+        <v>LK-8920</v>
       </c>
       <c r="E49" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn- 2000W LK-8920</v>
       </c>
       <c r="F49">
-        <v>375000</v>
+        <v>690000</v>
       </c>
       <c r="G49">
-        <v>750000</v>
+        <v>1290000</v>
       </c>
       <c r="H49">
-        <v>788000</v>
+        <v>1354500</v>
       </c>
       <c r="I49">
-        <v>946000</v>
+        <v>1626000</v>
       </c>
       <c r="J49">
-        <v>375000</v>
+        <v>600000</v>
       </c>
       <c r="K49" t="str">
-        <v>50.0%</v>
+        <v>46.5%</v>
       </c>
     </row>
     <row r="50">
@@ -2134,34 +2134,34 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C50" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-036A</v>
+        <v>LK-8818</v>
       </c>
       <c r="E50" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Nồi cơm cao tần LK-8818</v>
       </c>
       <c r="F50">
-        <v>515000</v>
+        <v>1790000</v>
       </c>
       <c r="G50">
-        <v>891000</v>
+        <v>3400000</v>
       </c>
       <c r="H50">
-        <v>936000</v>
+        <v>3570000</v>
       </c>
       <c r="I50">
-        <v>1124000</v>
+        <v>4284000</v>
       </c>
       <c r="J50">
-        <v>376000</v>
+        <v>1610000</v>
       </c>
       <c r="K50" t="str">
-        <v>42.2%</v>
+        <v>47.4%</v>
       </c>
     </row>
     <row r="51">
@@ -2169,34 +2169,34 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C51" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0324</v>
+        <v>LK-8618</v>
       </c>
       <c r="E51" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Nồi cơm tách đường LK-8618</v>
       </c>
       <c r="F51">
-        <v>245000</v>
+        <v>1300000</v>
       </c>
       <c r="G51">
-        <v>441000</v>
+        <v>2490000</v>
       </c>
       <c r="H51">
-        <v>464000</v>
+        <v>2614500</v>
       </c>
       <c r="I51">
-        <v>557000</v>
+        <v>3138000</v>
       </c>
       <c r="J51">
-        <v>196000</v>
+        <v>1190000</v>
       </c>
       <c r="K51" t="str">
-        <v>44.4%</v>
+        <v>47.8%</v>
       </c>
     </row>
     <row r="52">
@@ -2207,31 +2207,31 @@
         <v>Takin</v>
       </c>
       <c r="C52" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0348A</v>
+        <v>TK-2201</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F52">
-        <v>580000</v>
+        <v>265000</v>
       </c>
       <c r="G52">
-        <v>1044000</v>
+        <v>467000</v>
       </c>
       <c r="H52">
-        <v>1097000</v>
+        <v>491000</v>
       </c>
       <c r="I52">
-        <v>1317000</v>
+        <v>590000</v>
       </c>
       <c r="J52">
-        <v>464000</v>
+        <v>202000</v>
       </c>
       <c r="K52" t="str">
-        <v>44.4%</v>
+        <v>43.3%</v>
       </c>
     </row>
     <row r="53">
@@ -2242,31 +2242,31 @@
         <v>Takin</v>
       </c>
       <c r="C53" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0369</v>
+        <v>TK-2662</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F53">
-        <v>535000</v>
+        <v>320000</v>
       </c>
       <c r="G53">
-        <v>969000</v>
+        <v>590000</v>
       </c>
       <c r="H53">
-        <v>1018000</v>
+        <v>620000</v>
       </c>
       <c r="I53">
-        <v>1222000</v>
+        <v>744000</v>
       </c>
       <c r="J53">
-        <v>434000</v>
+        <v>270000</v>
       </c>
       <c r="K53" t="str">
-        <v>44.8%</v>
+        <v>45.8%</v>
       </c>
     </row>
     <row r="54">
@@ -2277,31 +2277,31 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-0488</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E54" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F54">
-        <v>810000</v>
+        <v>351000</v>
       </c>
       <c r="G54">
-        <v>1469000</v>
+        <v>630000</v>
       </c>
       <c r="H54">
-        <v>1543000</v>
+        <v>662000</v>
       </c>
       <c r="I54">
-        <v>1852000</v>
+        <v>795000</v>
       </c>
       <c r="J54">
-        <v>659000</v>
+        <v>279000</v>
       </c>
       <c r="K54" t="str">
-        <v>44.9%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="55">
@@ -2312,31 +2312,31 @@
         <v>Takin</v>
       </c>
       <c r="C55" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>CHẢO</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-468</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F55">
-        <v>452000</v>
+        <v>375000</v>
       </c>
       <c r="G55">
-        <v>900000</v>
+        <v>750000</v>
       </c>
       <c r="H55">
-        <v>945000</v>
+        <v>788000</v>
       </c>
       <c r="I55">
-        <v>1134000</v>
+        <v>946000</v>
       </c>
       <c r="J55">
-        <v>448000</v>
+        <v>375000</v>
       </c>
       <c r="K55" t="str">
-        <v>49.8%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="56">
@@ -2347,31 +2347,31 @@
         <v>Takin</v>
       </c>
       <c r="C56" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-469</v>
+        <v>TK-036A</v>
       </c>
       <c r="E56" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F56">
-        <v>615000</v>
+        <v>515000</v>
       </c>
       <c r="G56">
-        <v>1050000</v>
+        <v>891000</v>
       </c>
       <c r="H56">
-        <v>1103000</v>
+        <v>936000</v>
       </c>
       <c r="I56">
-        <v>1324000</v>
+        <v>1124000</v>
       </c>
       <c r="J56">
-        <v>435000</v>
+        <v>376000</v>
       </c>
       <c r="K56" t="str">
-        <v>41.4%</v>
+        <v>42.2%</v>
       </c>
     </row>
     <row r="57">
@@ -2382,31 +2382,31 @@
         <v>Takin</v>
       </c>
       <c r="C57" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1002</v>
+        <v>TK-0324</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F57">
-        <v>158000</v>
+        <v>245000</v>
       </c>
       <c r="G57">
-        <v>270000</v>
+        <v>441000</v>
       </c>
       <c r="H57">
-        <v>284000</v>
+        <v>464000</v>
       </c>
       <c r="I57">
-        <v>341000</v>
+        <v>557000</v>
       </c>
       <c r="J57">
-        <v>112000</v>
+        <v>196000</v>
       </c>
       <c r="K57" t="str">
-        <v>41.5%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="58">
@@ -2417,43 +2417,253 @@
         <v>Takin</v>
       </c>
       <c r="C58" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D58" t="str">
+        <v>TK-0348A</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+      </c>
+      <c r="F58">
+        <v>580000</v>
+      </c>
+      <c r="G58">
+        <v>1044000</v>
+      </c>
+      <c r="H58">
+        <v>1097000</v>
+      </c>
+      <c r="I58">
+        <v>1317000</v>
+      </c>
+      <c r="J58">
+        <v>464000</v>
+      </c>
+      <c r="K58" t="str">
+        <v>44.4%</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C59" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D59" t="str">
+        <v>TK-0369</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F59">
+        <v>535000</v>
+      </c>
+      <c r="G59">
+        <v>969000</v>
+      </c>
+      <c r="H59">
+        <v>1018000</v>
+      </c>
+      <c r="I59">
+        <v>1222000</v>
+      </c>
+      <c r="J59">
+        <v>434000</v>
+      </c>
+      <c r="K59" t="str">
+        <v>44.8%</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C60" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D60" t="str">
+        <v>TK-0488</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F60">
+        <v>810000</v>
+      </c>
+      <c r="G60">
+        <v>1469000</v>
+      </c>
+      <c r="H60">
+        <v>1543000</v>
+      </c>
+      <c r="I60">
+        <v>1852000</v>
+      </c>
+      <c r="J60">
+        <v>659000</v>
+      </c>
+      <c r="K60" t="str">
+        <v>44.9%</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C61" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D61" t="str">
+        <v>TK-468</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F61">
+        <v>452000</v>
+      </c>
+      <c r="G61">
+        <v>900000</v>
+      </c>
+      <c r="H61">
+        <v>945000</v>
+      </c>
+      <c r="I61">
+        <v>1134000</v>
+      </c>
+      <c r="J61">
+        <v>448000</v>
+      </c>
+      <c r="K61" t="str">
+        <v>49.8%</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C62" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D62" t="str">
+        <v>TK-469</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F62">
+        <v>615000</v>
+      </c>
+      <c r="G62">
+        <v>1050000</v>
+      </c>
+      <c r="H62">
+        <v>1103000</v>
+      </c>
+      <c r="I62">
+        <v>1324000</v>
+      </c>
+      <c r="J62">
+        <v>435000</v>
+      </c>
+      <c r="K62" t="str">
+        <v>41.4%</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D63" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F63">
+        <v>158000</v>
+      </c>
+      <c r="G63">
+        <v>270000</v>
+      </c>
+      <c r="H63">
+        <v>284000</v>
+      </c>
+      <c r="I63">
+        <v>341000</v>
+      </c>
+      <c r="J63">
+        <v>112000</v>
+      </c>
+      <c r="K63" t="str">
+        <v>41.5%</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C64" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D64" t="str">
         <v>TK-1003</v>
       </c>
-      <c r="E58" t="str">
+      <c r="E64" t="str">
         <v>Bộ đèn sưởi 3 bóng Takin</v>
       </c>
-      <c r="F58">
+      <c r="F64">
         <v>194000</v>
       </c>
-      <c r="G58">
+      <c r="G64">
         <v>330000</v>
       </c>
-      <c r="H58">
+      <c r="H64">
         <v>347000</v>
       </c>
-      <c r="I58">
+      <c r="I64">
         <v>417000</v>
       </c>
-      <c r="J58">
+      <c r="J64">
         <v>136000</v>
       </c>
-      <c r="K58" t="str">
+      <c r="K64" t="str">
         <v>41.2%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K64"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N64"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -3848,37 +4058,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1003</v>
+        <v>LK-6886</v>
       </c>
       <c r="E32" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo Model: LK 6886</v>
       </c>
       <c r="F32">
-        <v>167990</v>
+        <v>620000</v>
       </c>
       <c r="G32">
-        <v>197000</v>
+        <v>770000</v>
       </c>
       <c r="H32">
-        <v>354000</v>
+        <v>1490000</v>
       </c>
       <c r="I32">
-        <v>157000</v>
+        <v>720000</v>
       </c>
       <c r="J32" t="str">
-        <v>44.4%</v>
+        <v>48.3%</v>
       </c>
       <c r="K32">
-        <v>372000</v>
+        <v>1565000</v>
       </c>
       <c r="L32">
-        <v>18000</v>
+        <v>75000</v>
       </c>
       <c r="M32" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N32">
-        <v>447000</v>
+        <v>1878000</v>
       </c>
     </row>
     <row r="33">
@@ -3892,37 +4102,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E33" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F33">
-        <v>795408</v>
+        <v>160000</v>
       </c>
       <c r="G33">
-        <v>1020000</v>
+        <v>210000</v>
       </c>
       <c r="H33">
-        <v>1890000</v>
+        <v>399000</v>
       </c>
       <c r="I33">
-        <v>870000</v>
+        <v>189000</v>
       </c>
       <c r="J33" t="str">
-        <v>46.0%</v>
+        <v>47.4%</v>
       </c>
       <c r="K33">
-        <v>1985000</v>
+        <v>419000</v>
       </c>
       <c r="L33">
-        <v>95000</v>
+        <v>20000</v>
       </c>
       <c r="M33" t="str">
         <v>5.0%</v>
       </c>
       <c r="N33">
-        <v>2382000</v>
+        <v>503000</v>
       </c>
     </row>
     <row r="34">
@@ -3936,37 +4146,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E34" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F34">
-        <v>306020</v>
+        <v>795408</v>
       </c>
       <c r="G34">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="H34">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="I34">
-        <v>298000</v>
+        <v>870000</v>
       </c>
       <c r="J34" t="str">
-        <v>44.5%</v>
+        <v>46.0%</v>
       </c>
       <c r="K34">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
       <c r="L34">
-        <v>34000</v>
+        <v>95000</v>
       </c>
       <c r="M34" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N34">
-        <v>845000</v>
+        <v>2382000</v>
       </c>
     </row>
     <row r="35">
@@ -3980,37 +4190,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E35" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F35">
-        <v>668157</v>
+        <v>250000</v>
       </c>
       <c r="G35">
-        <v>780000</v>
+        <v>320000</v>
       </c>
       <c r="H35">
-        <v>1495000</v>
+        <v>620000</v>
       </c>
       <c r="I35">
-        <v>715000</v>
+        <v>300000</v>
       </c>
       <c r="J35" t="str">
-        <v>47.8%</v>
+        <v>48.4%</v>
       </c>
       <c r="K35">
-        <v>1570000</v>
+        <v>651000</v>
       </c>
       <c r="L35">
-        <v>75000</v>
+        <v>31000</v>
       </c>
       <c r="M35" t="str">
         <v>5.0%</v>
       </c>
       <c r="N35">
-        <v>1884000</v>
+        <v>782000</v>
       </c>
     </row>
     <row r="36">
@@ -4024,37 +4234,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E36" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F36">
-        <v>259549</v>
+        <v>668157</v>
       </c>
       <c r="G36">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="H36">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="I36">
-        <v>289000</v>
+        <v>715000</v>
       </c>
       <c r="J36" t="str">
-        <v>48.2%</v>
+        <v>47.8%</v>
       </c>
       <c r="K36">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
       <c r="L36">
-        <v>30000</v>
+        <v>75000</v>
       </c>
       <c r="M36" t="str">
         <v>5.0%</v>
       </c>
       <c r="N36">
-        <v>755000</v>
+        <v>1884000</v>
       </c>
     </row>
     <row r="37">
@@ -4068,37 +4278,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F37">
-        <v>828486</v>
+        <v>259549</v>
       </c>
       <c r="G37">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="H37">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="I37">
-        <v>880000</v>
+        <v>289000</v>
       </c>
       <c r="J37" t="str">
-        <v>46.8%</v>
+        <v>48.2%</v>
       </c>
       <c r="K37">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
       <c r="L37">
-        <v>94000</v>
+        <v>30000</v>
       </c>
       <c r="M37" t="str">
         <v>5.0%</v>
       </c>
       <c r="N37">
-        <v>2369000</v>
+        <v>755000</v>
       </c>
     </row>
     <row r="38">
@@ -4112,37 +4322,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F38">
-        <v>672571</v>
+        <v>828486</v>
       </c>
       <c r="G38">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H38">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="I38">
-        <v>690000</v>
+        <v>880000</v>
       </c>
       <c r="J38" t="str">
-        <v>46.3%</v>
+        <v>46.8%</v>
       </c>
       <c r="K38">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
       <c r="L38">
-        <v>75000</v>
+        <v>94000</v>
       </c>
       <c r="M38" t="str">
         <v>5.0%</v>
       </c>
       <c r="N38">
-        <v>1878000</v>
+        <v>2369000</v>
       </c>
     </row>
     <row r="39">
@@ -4156,37 +4366,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F39">
-        <v>399987</v>
+        <v>672571</v>
       </c>
       <c r="G39">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="H39">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="I39">
-        <v>440000</v>
+        <v>690000</v>
       </c>
       <c r="J39" t="str">
         <v>46.3%</v>
       </c>
       <c r="K39">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
       <c r="L39">
-        <v>48000</v>
+        <v>75000</v>
       </c>
       <c r="M39" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N39">
-        <v>1198000</v>
+        <v>1878000</v>
       </c>
     </row>
     <row r="40">
@@ -4200,13 +4410,13 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E40" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F40">
-        <v>389541</v>
+        <v>399987</v>
       </c>
       <c r="G40">
         <v>510000</v>
@@ -4244,37 +4454,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E41" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F41">
-        <v>468762</v>
+        <v>389541</v>
       </c>
       <c r="G41">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="H41">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="I41">
-        <v>590000</v>
+        <v>440000</v>
       </c>
       <c r="J41" t="str">
-        <v>49.6%</v>
+        <v>46.3%</v>
       </c>
       <c r="K41">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
       <c r="L41">
-        <v>60000</v>
+        <v>48000</v>
       </c>
       <c r="M41" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N41">
-        <v>1500000</v>
+        <v>1198000</v>
       </c>
     </row>
     <row r="42">
@@ -4288,37 +4498,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F42">
-        <v>200752</v>
+        <v>468762</v>
       </c>
       <c r="G42">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="H42">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="I42">
-        <v>230000</v>
+        <v>590000</v>
       </c>
       <c r="J42" t="str">
-        <v>46.9%</v>
+        <v>49.6%</v>
       </c>
       <c r="K42">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
       <c r="L42">
-        <v>25000</v>
+        <v>60000</v>
       </c>
       <c r="M42" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N42">
-        <v>618000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="43">
@@ -4332,37 +4542,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E43" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F43">
-        <v>550047</v>
+        <v>200752</v>
       </c>
       <c r="G43">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="H43">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="I43">
-        <v>605000</v>
+        <v>230000</v>
       </c>
       <c r="J43" t="str">
         <v>46.9%</v>
       </c>
       <c r="K43">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
       <c r="L43">
-        <v>65000</v>
+        <v>25000</v>
       </c>
       <c r="M43" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N43">
-        <v>1626000</v>
+        <v>618000</v>
       </c>
     </row>
     <row r="44">
@@ -4376,37 +4586,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E44" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F44">
-        <v>545604</v>
+        <v>550047</v>
       </c>
       <c r="G44">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="H44">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="I44">
-        <v>530000</v>
+        <v>605000</v>
       </c>
       <c r="J44" t="str">
-        <v>44.5%</v>
+        <v>46.9%</v>
       </c>
       <c r="K44">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
       <c r="L44">
-        <v>60000</v>
+        <v>65000</v>
       </c>
       <c r="M44" t="str">
         <v>5.0%</v>
       </c>
       <c r="N44">
-        <v>1500000</v>
+        <v>1626000</v>
       </c>
     </row>
     <row r="45">
@@ -4420,37 +4630,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E45" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F45">
-        <v>936250</v>
+        <v>545604</v>
       </c>
       <c r="G45">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="H45">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="I45">
-        <v>1060000</v>
+        <v>530000</v>
       </c>
       <c r="J45" t="str">
-        <v>48.4%</v>
+        <v>44.5%</v>
       </c>
       <c r="K45">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
       <c r="L45">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="M45" t="str">
         <v>5.0%</v>
       </c>
       <c r="N45">
-        <v>2760000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="46">
@@ -4458,43 +4668,43 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C46" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E46" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F46">
-        <v>203634</v>
+        <v>936250</v>
       </c>
       <c r="G46">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="H46">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="I46">
-        <v>202000</v>
+        <v>1060000</v>
       </c>
       <c r="J46" t="str">
-        <v>43.3%</v>
+        <v>48.4%</v>
       </c>
       <c r="K46">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
       <c r="L46">
-        <v>24000</v>
+        <v>110000</v>
       </c>
       <c r="M46" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N46">
-        <v>590000</v>
+        <v>2760000</v>
       </c>
     </row>
     <row r="47">
@@ -4502,43 +4712,43 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C47" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2662</v>
+        <v>LK-8989</v>
       </c>
       <c r="E47" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>Bếp từ đơn -2200W LK-8989</v>
       </c>
       <c r="F47">
-        <v>238375</v>
+        <v>650000</v>
       </c>
       <c r="G47">
-        <v>320000</v>
+        <v>790000</v>
       </c>
       <c r="H47">
-        <v>590000</v>
+        <v>1490000</v>
       </c>
       <c r="I47">
-        <v>270000</v>
+        <v>700000</v>
       </c>
       <c r="J47" t="str">
-        <v>45.8%</v>
+        <v>47.0%</v>
       </c>
       <c r="K47">
-        <v>620000</v>
+        <v>1565000</v>
       </c>
       <c r="L47">
-        <v>30000</v>
+        <v>75000</v>
       </c>
       <c r="M47" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N47">
-        <v>744000</v>
+        <v>1878000</v>
       </c>
     </row>
     <row r="48">
@@ -4546,43 +4756,43 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C48" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-2882C</v>
+        <v>LK-8924</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn -2400W LK-8924</v>
       </c>
       <c r="F48">
-        <v>266199</v>
+        <v>715000</v>
       </c>
       <c r="G48">
-        <v>351000</v>
+        <v>850000</v>
       </c>
       <c r="H48">
-        <v>630000</v>
+        <v>1590000</v>
       </c>
       <c r="I48">
-        <v>279000</v>
+        <v>740000</v>
       </c>
       <c r="J48" t="str">
-        <v>44.3%</v>
+        <v>46.5%</v>
       </c>
       <c r="K48">
-        <v>662000</v>
+        <v>1670000</v>
       </c>
       <c r="L48">
-        <v>32000</v>
+        <v>80000</v>
       </c>
       <c r="M48" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N48">
-        <v>795000</v>
+        <v>2004000</v>
       </c>
     </row>
     <row r="49">
@@ -4590,43 +4800,43 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C49" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-3030C</v>
+        <v>LK-8920</v>
       </c>
       <c r="E49" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn- 2000W LK-8920</v>
       </c>
       <c r="F49">
-        <v>290175</v>
+        <v>556000</v>
       </c>
       <c r="G49">
-        <v>375000</v>
+        <v>690000</v>
       </c>
       <c r="H49">
-        <v>750000</v>
+        <v>1290000</v>
       </c>
       <c r="I49">
-        <v>375000</v>
+        <v>600000</v>
       </c>
       <c r="J49" t="str">
-        <v>50.0%</v>
+        <v>46.5%</v>
       </c>
       <c r="K49">
-        <v>788000</v>
+        <v>1355000</v>
       </c>
       <c r="L49">
-        <v>38000</v>
+        <v>65000</v>
       </c>
       <c r="M49" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N49">
-        <v>946000</v>
+        <v>1626000</v>
       </c>
     </row>
     <row r="50">
@@ -4634,43 +4844,43 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C50" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-036A</v>
+        <v>LK-8818</v>
       </c>
       <c r="E50" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Nồi cơm cao tần LK-8818</v>
       </c>
       <c r="F50">
-        <v>433985</v>
+        <v>1400000</v>
       </c>
       <c r="G50">
-        <v>515000</v>
+        <v>1790000</v>
       </c>
       <c r="H50">
-        <v>891000</v>
+        <v>3400000</v>
       </c>
       <c r="I50">
-        <v>376000</v>
+        <v>1610000</v>
       </c>
       <c r="J50" t="str">
-        <v>42.2%</v>
+        <v>47.4%</v>
       </c>
       <c r="K50">
-        <v>936000</v>
+        <v>3570000</v>
       </c>
       <c r="L50">
-        <v>45000</v>
+        <v>170000</v>
       </c>
       <c r="M50" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N50">
-        <v>1124000</v>
+        <v>4284000</v>
       </c>
     </row>
     <row r="51">
@@ -4678,43 +4888,43 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C51" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0324</v>
+        <v>LK-8618</v>
       </c>
       <c r="E51" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Nồi cơm tách đường LK-8618</v>
       </c>
       <c r="F51">
-        <v>188524</v>
+        <v>1043000</v>
       </c>
       <c r="G51">
-        <v>245000</v>
+        <v>1300000</v>
       </c>
       <c r="H51">
-        <v>441000</v>
+        <v>2490000</v>
       </c>
       <c r="I51">
-        <v>196000</v>
+        <v>1190000</v>
       </c>
       <c r="J51" t="str">
-        <v>44.4%</v>
+        <v>47.8%</v>
       </c>
       <c r="K51">
-        <v>464000</v>
+        <v>2615000</v>
       </c>
       <c r="L51">
-        <v>23000</v>
+        <v>125000</v>
       </c>
       <c r="M51" t="str">
-        <v>5.2%</v>
+        <v>5.0%</v>
       </c>
       <c r="N51">
-        <v>557000</v>
+        <v>3138000</v>
       </c>
     </row>
     <row r="52">
@@ -4725,40 +4935,40 @@
         <v>Takin</v>
       </c>
       <c r="C52" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0348A</v>
+        <v>TK-2201</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F52">
-        <v>492000</v>
+        <v>203634</v>
       </c>
       <c r="G52">
-        <v>580000</v>
+        <v>265000</v>
       </c>
       <c r="H52">
-        <v>1044000</v>
+        <v>467000</v>
       </c>
       <c r="I52">
-        <v>464000</v>
+        <v>202000</v>
       </c>
       <c r="J52" t="str">
-        <v>44.4%</v>
+        <v>43.3%</v>
       </c>
       <c r="K52">
-        <v>1097000</v>
+        <v>491000</v>
       </c>
       <c r="L52">
-        <v>53000</v>
+        <v>24000</v>
       </c>
       <c r="M52" t="str">
         <v>5.1%</v>
       </c>
       <c r="N52">
-        <v>1317000</v>
+        <v>590000</v>
       </c>
     </row>
     <row r="53">
@@ -4769,40 +4979,40 @@
         <v>Takin</v>
       </c>
       <c r="C53" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0369</v>
+        <v>TK-2662</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F53">
-        <v>419848</v>
+        <v>238375</v>
       </c>
       <c r="G53">
-        <v>535000</v>
+        <v>320000</v>
       </c>
       <c r="H53">
-        <v>969000</v>
+        <v>590000</v>
       </c>
       <c r="I53">
-        <v>434000</v>
+        <v>270000</v>
       </c>
       <c r="J53" t="str">
-        <v>44.8%</v>
+        <v>45.8%</v>
       </c>
       <c r="K53">
-        <v>1018000</v>
+        <v>620000</v>
       </c>
       <c r="L53">
-        <v>49000</v>
+        <v>30000</v>
       </c>
       <c r="M53" t="str">
         <v>5.1%</v>
       </c>
       <c r="N53">
-        <v>1222000</v>
+        <v>744000</v>
       </c>
     </row>
     <row r="54">
@@ -4813,40 +5023,40 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-0488</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E54" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F54">
-        <v>672571</v>
+        <v>266199</v>
       </c>
       <c r="G54">
-        <v>810000</v>
+        <v>351000</v>
       </c>
       <c r="H54">
-        <v>1469000</v>
+        <v>630000</v>
       </c>
       <c r="I54">
-        <v>659000</v>
+        <v>279000</v>
       </c>
       <c r="J54" t="str">
-        <v>44.9%</v>
+        <v>44.3%</v>
       </c>
       <c r="K54">
-        <v>1543000</v>
+        <v>662000</v>
       </c>
       <c r="L54">
-        <v>74000</v>
+        <v>32000</v>
       </c>
       <c r="M54" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N54">
-        <v>1852000</v>
+        <v>795000</v>
       </c>
     </row>
     <row r="55">
@@ -4857,40 +5067,40 @@
         <v>Takin</v>
       </c>
       <c r="C55" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>CHẢO</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-468</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F55">
-        <v>366857</v>
+        <v>290175</v>
       </c>
       <c r="G55">
-        <v>452000</v>
+        <v>375000</v>
       </c>
       <c r="H55">
-        <v>900000</v>
+        <v>750000</v>
       </c>
       <c r="I55">
-        <v>448000</v>
+        <v>375000</v>
       </c>
       <c r="J55" t="str">
-        <v>49.8%</v>
+        <v>50.0%</v>
       </c>
       <c r="K55">
-        <v>945000</v>
+        <v>788000</v>
       </c>
       <c r="L55">
-        <v>45000</v>
+        <v>38000</v>
       </c>
       <c r="M55" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N55">
-        <v>1134000</v>
+        <v>946000</v>
       </c>
     </row>
     <row r="56">
@@ -4901,40 +5111,40 @@
         <v>Takin</v>
       </c>
       <c r="C56" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-469</v>
+        <v>TK-036A</v>
       </c>
       <c r="E56" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F56">
-        <v>468762</v>
+        <v>433985</v>
       </c>
       <c r="G56">
-        <v>615000</v>
+        <v>515000</v>
       </c>
       <c r="H56">
-        <v>1050000</v>
+        <v>891000</v>
       </c>
       <c r="I56">
-        <v>435000</v>
+        <v>376000</v>
       </c>
       <c r="J56" t="str">
-        <v>41.4%</v>
+        <v>42.2%</v>
       </c>
       <c r="K56">
-        <v>1103000</v>
+        <v>936000</v>
       </c>
       <c r="L56">
-        <v>53000</v>
+        <v>45000</v>
       </c>
       <c r="M56" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N56">
-        <v>1324000</v>
+        <v>1124000</v>
       </c>
     </row>
     <row r="57">
@@ -4945,40 +5155,40 @@
         <v>Takin</v>
       </c>
       <c r="C57" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1002</v>
+        <v>TK-0324</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F57">
-        <v>128400</v>
+        <v>188524</v>
       </c>
       <c r="G57">
-        <v>158000</v>
+        <v>245000</v>
       </c>
       <c r="H57">
-        <v>270000</v>
+        <v>441000</v>
       </c>
       <c r="I57">
-        <v>112000</v>
+        <v>196000</v>
       </c>
       <c r="J57" t="str">
-        <v>41.5%</v>
+        <v>44.4%</v>
       </c>
       <c r="K57">
-        <v>284000</v>
+        <v>464000</v>
       </c>
       <c r="L57">
-        <v>14000</v>
+        <v>23000</v>
       </c>
       <c r="M57" t="str">
         <v>5.2%</v>
       </c>
       <c r="N57">
-        <v>341000</v>
+        <v>557000</v>
       </c>
     </row>
     <row r="58">
@@ -4989,52 +5199,316 @@
         <v>Takin</v>
       </c>
       <c r="C58" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D58" t="str">
+        <v>TK-0348A</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+      </c>
+      <c r="F58">
+        <v>492000</v>
+      </c>
+      <c r="G58">
+        <v>580000</v>
+      </c>
+      <c r="H58">
+        <v>1044000</v>
+      </c>
+      <c r="I58">
+        <v>464000</v>
+      </c>
+      <c r="J58" t="str">
+        <v>44.4%</v>
+      </c>
+      <c r="K58">
+        <v>1097000</v>
+      </c>
+      <c r="L58">
+        <v>53000</v>
+      </c>
+      <c r="M58" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N58">
+        <v>1317000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C59" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D59" t="str">
+        <v>TK-0369</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F59">
+        <v>419848</v>
+      </c>
+      <c r="G59">
+        <v>535000</v>
+      </c>
+      <c r="H59">
+        <v>969000</v>
+      </c>
+      <c r="I59">
+        <v>434000</v>
+      </c>
+      <c r="J59" t="str">
+        <v>44.8%</v>
+      </c>
+      <c r="K59">
+        <v>1018000</v>
+      </c>
+      <c r="L59">
+        <v>49000</v>
+      </c>
+      <c r="M59" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N59">
+        <v>1222000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C60" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D60" t="str">
+        <v>TK-0488</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F60">
+        <v>672571</v>
+      </c>
+      <c r="G60">
+        <v>810000</v>
+      </c>
+      <c r="H60">
+        <v>1469000</v>
+      </c>
+      <c r="I60">
+        <v>659000</v>
+      </c>
+      <c r="J60" t="str">
+        <v>44.9%</v>
+      </c>
+      <c r="K60">
+        <v>1543000</v>
+      </c>
+      <c r="L60">
+        <v>74000</v>
+      </c>
+      <c r="M60" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N60">
+        <v>1852000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C61" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D61" t="str">
+        <v>TK-468</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F61">
+        <v>366857</v>
+      </c>
+      <c r="G61">
+        <v>452000</v>
+      </c>
+      <c r="H61">
+        <v>900000</v>
+      </c>
+      <c r="I61">
+        <v>448000</v>
+      </c>
+      <c r="J61" t="str">
+        <v>49.8%</v>
+      </c>
+      <c r="K61">
+        <v>945000</v>
+      </c>
+      <c r="L61">
+        <v>45000</v>
+      </c>
+      <c r="M61" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N61">
+        <v>1134000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C62" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D62" t="str">
+        <v>TK-469</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F62">
+        <v>468762</v>
+      </c>
+      <c r="G62">
+        <v>615000</v>
+      </c>
+      <c r="H62">
+        <v>1050000</v>
+      </c>
+      <c r="I62">
+        <v>435000</v>
+      </c>
+      <c r="J62" t="str">
+        <v>41.4%</v>
+      </c>
+      <c r="K62">
+        <v>1103000</v>
+      </c>
+      <c r="L62">
+        <v>53000</v>
+      </c>
+      <c r="M62" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N62">
+        <v>1324000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D63" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F63">
+        <v>128400</v>
+      </c>
+      <c r="G63">
+        <v>158000</v>
+      </c>
+      <c r="H63">
+        <v>270000</v>
+      </c>
+      <c r="I63">
+        <v>112000</v>
+      </c>
+      <c r="J63" t="str">
+        <v>41.5%</v>
+      </c>
+      <c r="K63">
+        <v>284000</v>
+      </c>
+      <c r="L63">
+        <v>14000</v>
+      </c>
+      <c r="M63" t="str">
+        <v>5.2%</v>
+      </c>
+      <c r="N63">
+        <v>341000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C64" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D64" t="str">
         <v>TK-1003</v>
       </c>
-      <c r="E58" t="str">
+      <c r="E64" t="str">
         <v>Bộ đèn sưởi 3 bóng Takin</v>
       </c>
-      <c r="F58">
+      <c r="F64">
         <v>157290</v>
       </c>
-      <c r="G58">
+      <c r="G64">
         <v>194000</v>
       </c>
-      <c r="H58">
+      <c r="H64">
         <v>330000</v>
       </c>
-      <c r="I58">
+      <c r="I64">
         <v>136000</v>
       </c>
-      <c r="J58" t="str">
+      <c r="J64" t="str">
         <v>41.2%</v>
       </c>
-      <c r="K58">
+      <c r="K64">
         <v>347000</v>
       </c>
-      <c r="L58">
+      <c r="L64">
         <v>17000</v>
       </c>
-      <c r="M58" t="str">
+      <c r="M64" t="str">
         <v>5.2%</v>
       </c>
-      <c r="N58">
+      <c r="N64">
         <v>417000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N64"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L64"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -6239,16 +6713,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1003</v>
+        <v>LK-6886</v>
       </c>
       <c r="E32" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Tủ sấy quần áo Model: LK 6886</v>
       </c>
       <c r="F32">
-        <v>197000</v>
+        <v>770000</v>
       </c>
       <c r="G32">
-        <v>197000</v>
+        <v>770000</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -6260,10 +6734,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K32">
-        <v>354000</v>
+        <v>1490000</v>
       </c>
       <c r="L32">
-        <v>372000</v>
+        <v>1564500</v>
       </c>
     </row>
     <row r="33">
@@ -6277,31 +6751,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1030</v>
+        <v>LK-1003</v>
       </c>
       <c r="E33" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F33">
-        <v>1020000</v>
+        <v>197000</v>
       </c>
       <c r="G33">
-        <v>1020000</v>
+        <v>210000</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>13000</v>
       </c>
       <c r="I33" t="str">
-        <v>0.0%</v>
+        <v>6.6%</v>
       </c>
       <c r="J33" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K33">
-        <v>1890000</v>
+        <v>399000</v>
       </c>
       <c r="L33">
-        <v>1985000</v>
+        <v>418950</v>
       </c>
     </row>
     <row r="34">
@@ -6315,16 +6789,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1033</v>
+        <v>LK-1030</v>
       </c>
       <c r="E34" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F34">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="G34">
-        <v>372000</v>
+        <v>1020000</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -6336,10 +6810,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K34">
-        <v>670000</v>
+        <v>1890000</v>
       </c>
       <c r="L34">
-        <v>704000</v>
+        <v>1985000</v>
       </c>
     </row>
     <row r="35">
@@ -6353,31 +6827,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1050</v>
+        <v>LK-1033</v>
       </c>
       <c r="E35" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F35">
-        <v>890000</v>
+        <v>372000</v>
       </c>
       <c r="G35">
-        <v>780000</v>
+        <v>320000</v>
       </c>
       <c r="H35">
-        <v>-110000</v>
+        <v>-52000</v>
       </c>
       <c r="I35" t="str">
-        <v>-12.4%</v>
+        <v>-14.0%</v>
       </c>
       <c r="J35" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K35">
-        <v>1495000</v>
+        <v>620000</v>
       </c>
       <c r="L35">
-        <v>1570000</v>
+        <v>651000</v>
       </c>
     </row>
     <row r="36">
@@ -6391,31 +6865,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-1068</v>
+        <v>LK-1050</v>
       </c>
       <c r="E36" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F36">
-        <v>340000</v>
+        <v>890000</v>
       </c>
       <c r="G36">
-        <v>310000</v>
+        <v>780000</v>
       </c>
       <c r="H36">
-        <v>-30000</v>
+        <v>-110000</v>
       </c>
       <c r="I36" t="str">
-        <v>-8.8%</v>
+        <v>-12.4%</v>
       </c>
       <c r="J36" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K36">
-        <v>599000</v>
+        <v>1495000</v>
       </c>
       <c r="L36">
-        <v>629000</v>
+        <v>1570000</v>
       </c>
     </row>
     <row r="37">
@@ -6429,31 +6903,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4160</v>
+        <v>LK-1068</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F37">
-        <v>1080000</v>
+        <v>340000</v>
       </c>
       <c r="G37">
-        <v>1000000</v>
+        <v>310000</v>
       </c>
       <c r="H37">
-        <v>-80000</v>
+        <v>-30000</v>
       </c>
       <c r="I37" t="str">
-        <v>-7.4%</v>
+        <v>-8.8%</v>
       </c>
       <c r="J37" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K37">
-        <v>1880000</v>
+        <v>599000</v>
       </c>
       <c r="L37">
-        <v>1974000</v>
+        <v>629000</v>
       </c>
     </row>
     <row r="38">
@@ -6467,31 +6941,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4161</v>
+        <v>LK-4160</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F38">
-        <v>850000</v>
+        <v>1080000</v>
       </c>
       <c r="G38">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H38">
-        <v>-50000</v>
+        <v>-80000</v>
       </c>
       <c r="I38" t="str">
-        <v>-5.9%</v>
+        <v>-7.4%</v>
       </c>
       <c r="J38" t="str">
         <v>Giảm giá</v>
       </c>
       <c r="K38">
-        <v>1490000</v>
+        <v>1880000</v>
       </c>
       <c r="L38">
-        <v>1565000</v>
+        <v>1974000</v>
       </c>
     </row>
     <row r="39">
@@ -6505,31 +6979,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4161</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F39">
-        <v>510000</v>
+        <v>850000</v>
       </c>
       <c r="G39">
-        <v>510000</v>
+        <v>800000</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="I39" t="str">
-        <v>0.0%</v>
+        <v>-5.9%</v>
       </c>
       <c r="J39" t="str">
-        <v>Giữ nguyên</v>
+        <v>Giảm giá</v>
       </c>
       <c r="K39">
-        <v>950000</v>
+        <v>1490000</v>
       </c>
       <c r="L39">
-        <v>998000</v>
+        <v>1565000</v>
       </c>
     </row>
     <row r="40">
@@ -6543,10 +7017,10 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-4209</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E40" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F40">
         <v>510000</v>
@@ -6581,16 +7055,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-5301</v>
+        <v>LK-4209</v>
       </c>
       <c r="E41" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F41">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="G41">
-        <v>600000</v>
+        <v>510000</v>
       </c>
       <c r="H41">
         <v>0</v>
@@ -6602,10 +7076,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K41">
-        <v>1190000</v>
+        <v>950000</v>
       </c>
       <c r="L41">
-        <v>1250000</v>
+        <v>998000</v>
       </c>
     </row>
     <row r="42">
@@ -6619,16 +7093,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6015</v>
+        <v>LK-5301</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F42">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="G42">
-        <v>260000</v>
+        <v>600000</v>
       </c>
       <c r="H42">
         <v>0</v>
@@ -6640,10 +7114,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K42">
-        <v>490000</v>
+        <v>1190000</v>
       </c>
       <c r="L42">
-        <v>515000</v>
+        <v>1250000</v>
       </c>
     </row>
     <row r="43">
@@ -6657,16 +7131,16 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-6201</v>
+        <v>LK-6015</v>
       </c>
       <c r="E43" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F43">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="G43">
-        <v>685000</v>
+        <v>260000</v>
       </c>
       <c r="H43">
         <v>0</v>
@@ -6678,10 +7152,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K43">
-        <v>1290000</v>
+        <v>490000</v>
       </c>
       <c r="L43">
-        <v>1355000</v>
+        <v>515000</v>
       </c>
     </row>
     <row r="44">
@@ -6695,31 +7169,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-7812</v>
+        <v>LK-6201</v>
       </c>
       <c r="E44" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F44">
-        <v>710000</v>
+        <v>685000</v>
       </c>
       <c r="G44">
-        <v>660000</v>
+        <v>685000</v>
       </c>
       <c r="H44">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="I44" t="str">
-        <v>-7.0%</v>
+        <v>0.0%</v>
       </c>
       <c r="J44" t="str">
-        <v>Giảm giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K44">
-        <v>1190000</v>
+        <v>1290000</v>
       </c>
       <c r="L44">
-        <v>1250000</v>
+        <v>1355000</v>
       </c>
     </row>
     <row r="45">
@@ -6733,31 +7207,31 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D45" t="str">
-        <v>LK-9014</v>
+        <v>LK-7812</v>
       </c>
       <c r="E45" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F45">
-        <v>1130000</v>
+        <v>710000</v>
       </c>
       <c r="G45">
-        <v>1130000</v>
+        <v>660000</v>
       </c>
       <c r="H45">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="I45" t="str">
-        <v>0.0%</v>
+        <v>-7.0%</v>
       </c>
       <c r="J45" t="str">
-        <v>Giữ nguyên</v>
+        <v>Giảm giá</v>
       </c>
       <c r="K45">
-        <v>2190000</v>
+        <v>1190000</v>
       </c>
       <c r="L45">
-        <v>2300000</v>
+        <v>1250000</v>
       </c>
     </row>
     <row r="46">
@@ -6765,37 +7239,37 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C46" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2201</v>
+        <v>LK-9014</v>
       </c>
       <c r="E46" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F46">
-        <v>260000</v>
+        <v>1130000</v>
       </c>
       <c r="G46">
-        <v>265000</v>
+        <v>1130000</v>
       </c>
       <c r="H46">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="I46" t="str">
-        <v>1.9%</v>
+        <v>0.0%</v>
       </c>
       <c r="J46" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K46">
-        <v>467000</v>
+        <v>2190000</v>
       </c>
       <c r="L46">
-        <v>491000</v>
+        <v>2300000</v>
       </c>
     </row>
     <row r="47">
@@ -6803,37 +7277,37 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C47" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2662</v>
+        <v>LK-8989</v>
       </c>
       <c r="E47" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>Bếp từ đơn -2200W LK-8989</v>
       </c>
       <c r="F47">
-        <v>310000</v>
+        <v>790000</v>
       </c>
       <c r="G47">
-        <v>320000</v>
+        <v>790000</v>
       </c>
       <c r="H47">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I47" t="str">
-        <v>3.2%</v>
+        <v>0.0%</v>
       </c>
       <c r="J47" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K47">
-        <v>590000</v>
+        <v>1490000</v>
       </c>
       <c r="L47">
-        <v>620000</v>
+        <v>1564500</v>
       </c>
     </row>
     <row r="48">
@@ -6841,37 +7315,37 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C48" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-2882C</v>
+        <v>LK-8924</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn -2400W LK-8924</v>
       </c>
       <c r="F48">
-        <v>341000</v>
+        <v>850000</v>
       </c>
       <c r="G48">
-        <v>351000</v>
+        <v>850000</v>
       </c>
       <c r="H48">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I48" t="str">
-        <v>2.9%</v>
+        <v>0.0%</v>
       </c>
       <c r="J48" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K48">
-        <v>630000</v>
+        <v>1590000</v>
       </c>
       <c r="L48">
-        <v>662000</v>
+        <v>1669500</v>
       </c>
     </row>
     <row r="49">
@@ -6879,37 +7353,37 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C49" t="str">
-        <v>CHẢO</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-3030C</v>
+        <v>LK-8920</v>
       </c>
       <c r="E49" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Bếp từ đơn- 2000W LK-8920</v>
       </c>
       <c r="F49">
-        <v>360000</v>
+        <v>690000</v>
       </c>
       <c r="G49">
-        <v>375000</v>
+        <v>690000</v>
       </c>
       <c r="H49">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I49" t="str">
-        <v>4.2%</v>
+        <v>0.0%</v>
       </c>
       <c r="J49" t="str">
-        <v>Tăng giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K49">
-        <v>750000</v>
+        <v>1290000</v>
       </c>
       <c r="L49">
-        <v>788000</v>
+        <v>1354500</v>
       </c>
     </row>
     <row r="50">
@@ -6917,22 +7391,22 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C50" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-036A</v>
+        <v>LK-8818</v>
       </c>
       <c r="E50" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Nồi cơm cao tần LK-8818</v>
       </c>
       <c r="F50">
-        <v>515000</v>
+        <v>1790000</v>
       </c>
       <c r="G50">
-        <v>515000</v>
+        <v>1790000</v>
       </c>
       <c r="H50">
         <v>0</v>
@@ -6944,10 +7418,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K50">
-        <v>891000</v>
+        <v>3400000</v>
       </c>
       <c r="L50">
-        <v>936000</v>
+        <v>3570000</v>
       </c>
     </row>
     <row r="51">
@@ -6955,22 +7429,22 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>Takin</v>
+        <v>Lock&amp;King</v>
       </c>
       <c r="C51" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0324</v>
+        <v>LK-8618</v>
       </c>
       <c r="E51" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Nồi cơm tách đường LK-8618</v>
       </c>
       <c r="F51">
-        <v>245000</v>
+        <v>1300000</v>
       </c>
       <c r="G51">
-        <v>245000</v>
+        <v>1300000</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -6982,10 +7456,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K51">
-        <v>441000</v>
+        <v>2490000</v>
       </c>
       <c r="L51">
-        <v>464000</v>
+        <v>2614500</v>
       </c>
     </row>
     <row r="52">
@@ -6996,34 +7470,34 @@
         <v>Takin</v>
       </c>
       <c r="C52" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0348A</v>
+        <v>TK-2201</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F52">
-        <v>580000</v>
+        <v>260000</v>
       </c>
       <c r="G52">
-        <v>580000</v>
+        <v>265000</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="I52" t="str">
-        <v>0.0%</v>
+        <v>1.9%</v>
       </c>
       <c r="J52" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K52">
-        <v>1044000</v>
+        <v>467000</v>
       </c>
       <c r="L52">
-        <v>1097000</v>
+        <v>491000</v>
       </c>
     </row>
     <row r="53">
@@ -7034,34 +7508,34 @@
         <v>Takin</v>
       </c>
       <c r="C53" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0369</v>
+        <v>TK-2662</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F53">
-        <v>535000</v>
+        <v>310000</v>
       </c>
       <c r="G53">
-        <v>535000</v>
+        <v>320000</v>
       </c>
       <c r="H53">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I53" t="str">
-        <v>0.0%</v>
+        <v>3.2%</v>
       </c>
       <c r="J53" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K53">
-        <v>969000</v>
+        <v>590000</v>
       </c>
       <c r="L53">
-        <v>1018000</v>
+        <v>620000</v>
       </c>
     </row>
     <row r="54">
@@ -7072,34 +7546,34 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>CHẢO</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-0488</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E54" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F54">
-        <v>810000</v>
+        <v>341000</v>
       </c>
       <c r="G54">
-        <v>810000</v>
+        <v>351000</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I54" t="str">
-        <v>0.0%</v>
+        <v>2.9%</v>
       </c>
       <c r="J54" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K54">
-        <v>1469000</v>
+        <v>630000</v>
       </c>
       <c r="L54">
-        <v>1543000</v>
+        <v>662000</v>
       </c>
     </row>
     <row r="55">
@@ -7110,34 +7584,34 @@
         <v>Takin</v>
       </c>
       <c r="C55" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>CHẢO</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-468</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F55">
-        <v>452000</v>
+        <v>360000</v>
       </c>
       <c r="G55">
-        <v>452000</v>
+        <v>375000</v>
       </c>
       <c r="H55">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I55" t="str">
-        <v>0.0%</v>
+        <v>4.2%</v>
       </c>
       <c r="J55" t="str">
-        <v>Giữ nguyên</v>
+        <v>Tăng giá</v>
       </c>
       <c r="K55">
-        <v>900000</v>
+        <v>750000</v>
       </c>
       <c r="L55">
-        <v>945000</v>
+        <v>788000</v>
       </c>
     </row>
     <row r="56">
@@ -7148,19 +7622,19 @@
         <v>Takin</v>
       </c>
       <c r="C56" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-469</v>
+        <v>TK-036A</v>
       </c>
       <c r="E56" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F56">
-        <v>615000</v>
+        <v>515000</v>
       </c>
       <c r="G56">
-        <v>615000</v>
+        <v>515000</v>
       </c>
       <c r="H56">
         <v>0</v>
@@ -7172,10 +7646,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K56">
-        <v>1050000</v>
+        <v>891000</v>
       </c>
       <c r="L56">
-        <v>1103000</v>
+        <v>936000</v>
       </c>
     </row>
     <row r="57">
@@ -7186,19 +7660,19 @@
         <v>Takin</v>
       </c>
       <c r="C57" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1002</v>
+        <v>TK-0324</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F57">
-        <v>158000</v>
+        <v>245000</v>
       </c>
       <c r="G57">
-        <v>158000</v>
+        <v>245000</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -7210,10 +7684,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K57">
-        <v>270000</v>
+        <v>441000</v>
       </c>
       <c r="L57">
-        <v>284000</v>
+        <v>464000</v>
       </c>
     </row>
     <row r="58">
@@ -7224,19 +7698,19 @@
         <v>Takin</v>
       </c>
       <c r="C58" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D58" t="str">
-        <v>TK-1003</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E58" t="str">
-        <v>Bộ đèn sưởi 3 bóng Takin</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F58">
-        <v>194000</v>
+        <v>580000</v>
       </c>
       <c r="G58">
-        <v>194000</v>
+        <v>580000</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -7248,15 +7722,243 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K58">
+        <v>1044000</v>
+      </c>
+      <c r="L58">
+        <v>1097000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C59" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D59" t="str">
+        <v>TK-0369</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F59">
+        <v>535000</v>
+      </c>
+      <c r="G59">
+        <v>535000</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K59">
+        <v>969000</v>
+      </c>
+      <c r="L59">
+        <v>1018000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C60" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D60" t="str">
+        <v>TK-0488</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F60">
+        <v>810000</v>
+      </c>
+      <c r="G60">
+        <v>810000</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K60">
+        <v>1469000</v>
+      </c>
+      <c r="L60">
+        <v>1543000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C61" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D61" t="str">
+        <v>TK-468</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F61">
+        <v>452000</v>
+      </c>
+      <c r="G61">
+        <v>452000</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K61">
+        <v>900000</v>
+      </c>
+      <c r="L61">
+        <v>945000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C62" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D62" t="str">
+        <v>TK-469</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F62">
+        <v>615000</v>
+      </c>
+      <c r="G62">
+        <v>615000</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K62">
+        <v>1050000</v>
+      </c>
+      <c r="L62">
+        <v>1103000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D63" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F63">
+        <v>158000</v>
+      </c>
+      <c r="G63">
+        <v>158000</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J63" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K63">
+        <v>270000</v>
+      </c>
+      <c r="L63">
+        <v>284000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C64" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D64" t="str">
+        <v>TK-1003</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
+      </c>
+      <c r="F64">
+        <v>194000</v>
+      </c>
+      <c r="G64">
+        <v>194000</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K64">
         <v>330000</v>
       </c>
-      <c r="L58">
+      <c r="L64">
         <v>347000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: bo sung Sheet 4 BienDong_CapNhat_MoiNhat va tinh nang xuat nhat ky bien dong gia dot moi nhat
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Bang_Gia_Chuan_63_Ma" sheetId="1" r:id="rId1"/>
     <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
     <sheet name="BienDong_Gia_NPP" sheetId="3" r:id="rId3"/>
+    <sheet name="BienDong_CapNhat_MoiNhat" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -7961,4 +7962,567 @@
     <ignoredError numberStoredAsText="1" sqref="A1:L64"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S9"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="42.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="16.83203125" customWidth="1"/>
+    <col min="19" max="19" width="65.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Ngày Cập Nhật</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Loại Biến Động</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Model (Mã Sản Phẩm)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Tên Sản Phẩm</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Phân Loại</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Thương Hiệu</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Giá Vốn Cũ (VNĐ)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Giá Vốn Mới (VNĐ)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Giá NPP Online Cũ (VNĐ)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Giá NPP Online Mới (VNĐ)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Chênh Lệch NPP (VNĐ)</v>
+      </c>
+      <c r="M1" t="str">
+        <v>% Biến Động NPP</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Giá Facebook (VNĐ)</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Giá Sàn TMĐT (VNĐ)</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Giá Niêm Yết (VNĐ)</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Lợi Nhuận NPP (VNĐ)</v>
+      </c>
+      <c r="R1" t="str">
+        <v>% LN NPP / FB</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Ghi Chú Nghiệp Vụ</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D2" t="str">
+        <v>LK-8920</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Bếp từ đơn- 2000W LK-8920</v>
+      </c>
+      <c r="F2" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>556000</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>690000</v>
+      </c>
+      <c r="L2">
+        <v>690000</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N2">
+        <v>1290000</v>
+      </c>
+      <c r="O2">
+        <v>1354500</v>
+      </c>
+      <c r="P2">
+        <v>1626000</v>
+      </c>
+      <c r="Q2">
+        <v>600000</v>
+      </c>
+      <c r="R2" t="str">
+        <v>46.5%</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Bếp từ đơn 2000W mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D3" t="str">
+        <v>LK-8989</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Bếp từ đơn -2200W LK-8989</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>650000</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>790000</v>
+      </c>
+      <c r="L3">
+        <v>790000</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N3">
+        <v>1490000</v>
+      </c>
+      <c r="O3">
+        <v>1564500</v>
+      </c>
+      <c r="P3">
+        <v>1878000</v>
+      </c>
+      <c r="Q3">
+        <v>700000</v>
+      </c>
+      <c r="R3" t="str">
+        <v>47.0%</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Bếp từ đơn 2200W mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D4" t="str">
+        <v>LK-8924</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Bếp từ đơn -2400W LK-8924</v>
+      </c>
+      <c r="F4" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>715000</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>850000</v>
+      </c>
+      <c r="L4">
+        <v>850000</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N4">
+        <v>1590000</v>
+      </c>
+      <c r="O4">
+        <v>1669500</v>
+      </c>
+      <c r="P4">
+        <v>2004000</v>
+      </c>
+      <c r="Q4">
+        <v>740000</v>
+      </c>
+      <c r="R4" t="str">
+        <v>46.5%</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Bếp từ đơn 2400W mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LK-8818</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Nồi cơm cao tần LK-8818</v>
+      </c>
+      <c r="F5" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>1400000</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>1790000</v>
+      </c>
+      <c r="L5">
+        <v>1790000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N5">
+        <v>3400000</v>
+      </c>
+      <c r="O5">
+        <v>3570000</v>
+      </c>
+      <c r="P5">
+        <v>4284000</v>
+      </c>
+      <c r="Q5">
+        <v>1610000</v>
+      </c>
+      <c r="R5" t="str">
+        <v>47.4%</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Nồi cơm điện cao tần IH mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LK-8618</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Nồi cơm tách đường LK-8618</v>
+      </c>
+      <c r="F6" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1043000</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>1300000</v>
+      </c>
+      <c r="L6">
+        <v>1300000</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N6">
+        <v>2490000</v>
+      </c>
+      <c r="O6">
+        <v>2614500</v>
+      </c>
+      <c r="P6">
+        <v>3138000</v>
+      </c>
+      <c r="Q6">
+        <v>1190000</v>
+      </c>
+      <c r="R6" t="str">
+        <v>47.8%</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Nồi cơm điện tách đường mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MÃ MỚI BỔ SUNG</v>
+      </c>
+      <c r="D7" t="str">
+        <v>LK-6886</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Tủ sấy quần áo Model: LK 6886</v>
+      </c>
+      <c r="F7" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>620000</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>770000</v>
+      </c>
+      <c r="L7">
+        <v>770000</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Mới</v>
+      </c>
+      <c r="N7">
+        <v>1490000</v>
+      </c>
+      <c r="O7">
+        <v>1564500</v>
+      </c>
+      <c r="P7">
+        <v>1878000</v>
+      </c>
+      <c r="Q7">
+        <v>720000</v>
+      </c>
+      <c r="R7" t="str">
+        <v>48.3%</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Tủ sấy quần áo công suất lớn mới bổ sung danh mục</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ĐIỀU CHỈNH TĂNG GIÁ</v>
+      </c>
+      <c r="D8" t="str">
+        <v>LK-1003</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F8" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H8">
+        <v>133495</v>
+      </c>
+      <c r="I8">
+        <v>160000</v>
+      </c>
+      <c r="J8">
+        <v>197000</v>
+      </c>
+      <c r="K8">
+        <v>210000</v>
+      </c>
+      <c r="L8">
+        <v>13000</v>
+      </c>
+      <c r="M8" t="str">
+        <v>6.6%</v>
+      </c>
+      <c r="N8">
+        <v>399000</v>
+      </c>
+      <c r="O8">
+        <v>418950</v>
+      </c>
+      <c r="P8">
+        <v>503000</v>
+      </c>
+      <c r="Q8">
+        <v>189000</v>
+      </c>
+      <c r="R8" t="str">
+        <v>47.4%</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Đèn sưởi 3 bóng: Giá NPP tăng +13.000đ (+6.6%), vốn tăng +26.505đ</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ĐIỀU CHỈNH GIẢM GIÁ</v>
+      </c>
+      <c r="D9" t="str">
+        <v>LK-1033</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F9" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="H9">
+        <v>200000</v>
+      </c>
+      <c r="I9">
+        <v>250000</v>
+      </c>
+      <c r="J9">
+        <v>372000</v>
+      </c>
+      <c r="K9">
+        <v>320000</v>
+      </c>
+      <c r="L9">
+        <v>-52000</v>
+      </c>
+      <c r="M9" t="str">
+        <v>-14.0%</v>
+      </c>
+      <c r="N9">
+        <v>620000</v>
+      </c>
+      <c r="O9">
+        <v>651000</v>
+      </c>
+      <c r="P9">
+        <v>782000</v>
+      </c>
+      <c r="Q9">
+        <v>300000</v>
+      </c>
+      <c r="R9" t="str">
+        <v>48.4%</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Đèn sưởi 3 bóng: Giá NPP giảm -52.000đ (-14.0%), vốn tăng +50.000đ</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:S9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>